<commit_message>
Updating the model for Adrem
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B521"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,1042 +394,4162 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B2">
-        <v>513</v>
+        <v>428</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46277.01041666666</v>
+        <v>46278.01041666666</v>
       </c>
       <c r="B3">
-        <v>493</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46277.02083333334</v>
+        <v>46278.02083333334</v>
       </c>
       <c r="B4">
-        <v>529</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46277.03125</v>
+        <v>46278.03125</v>
       </c>
       <c r="B5">
-        <v>529</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46277.04166666666</v>
+        <v>46278.04166666666</v>
       </c>
       <c r="B6">
-        <v>514</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46277.05208333334</v>
+        <v>46278.05208333334</v>
       </c>
       <c r="B7">
-        <v>513</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46277.0625</v>
+        <v>46278.0625</v>
       </c>
       <c r="B8">
-        <v>513</v>
+        <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46277.07291666666</v>
+        <v>46278.07291666666</v>
       </c>
       <c r="B9">
-        <v>514</v>
+        <v>402</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46277.08333333334</v>
+        <v>46278.08333333334</v>
       </c>
       <c r="B10">
-        <v>513</v>
+        <v>415</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46277.09375</v>
+        <v>46278.09375</v>
       </c>
       <c r="B11">
-        <v>512</v>
+        <v>417</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46277.10416666666</v>
+        <v>46278.10416666666</v>
       </c>
       <c r="B12">
-        <v>513</v>
+        <v>416</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46277.11458333334</v>
+        <v>46278.11458333334</v>
       </c>
       <c r="B13">
-        <v>514</v>
+        <v>418</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46277.125</v>
+        <v>46278.125</v>
       </c>
       <c r="B14">
-        <v>519</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46277.13541666666</v>
+        <v>46278.13541666666</v>
       </c>
       <c r="B15">
-        <v>520</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46277.14583333334</v>
+        <v>46278.14583333334</v>
       </c>
       <c r="B16">
-        <v>508</v>
+        <v>335</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46277.15625</v>
+        <v>46278.15625</v>
       </c>
       <c r="B17">
-        <v>480</v>
+        <v>336</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46277.16666666666</v>
+        <v>46278.16666666666</v>
       </c>
       <c r="B18">
-        <v>480</v>
+        <v>389</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46277.17708333334</v>
+        <v>46278.17708333334</v>
       </c>
       <c r="B19">
-        <v>481</v>
+        <v>399</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46277.1875</v>
+        <v>46278.1875</v>
       </c>
       <c r="B20">
-        <v>481</v>
+        <v>400</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46277.19791666666</v>
+        <v>46278.19791666666</v>
       </c>
       <c r="B21">
-        <v>482</v>
+        <v>401</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46277.20833333334</v>
+        <v>46278.20833333334</v>
       </c>
       <c r="B22">
-        <v>484</v>
+        <v>441</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46277.21875</v>
+        <v>46278.21875</v>
       </c>
       <c r="B23">
-        <v>487</v>
+        <v>441</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46277.22916666666</v>
+        <v>46278.22916666666</v>
       </c>
       <c r="B24">
-        <v>525</v>
+        <v>433</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46277.23958333334</v>
+        <v>46278.23958333334</v>
       </c>
       <c r="B25">
-        <v>525</v>
+        <v>433</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46277.25</v>
+        <v>46278.25</v>
       </c>
       <c r="B26">
-        <v>520</v>
+        <v>447</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46277.26041666666</v>
+        <v>46278.26041666666</v>
       </c>
       <c r="B27">
-        <v>466</v>
+        <v>451</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46277.27083333334</v>
+        <v>46278.27083333334</v>
       </c>
       <c r="B28">
-        <v>464</v>
+        <v>452</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46277.28125</v>
+        <v>46278.28125</v>
       </c>
       <c r="B29">
-        <v>461</v>
+        <v>453</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46277.29166666666</v>
+        <v>46278.29166666666</v>
       </c>
       <c r="B30">
-        <v>470</v>
+        <v>443</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46277.30208333334</v>
+        <v>46278.30208333334</v>
       </c>
       <c r="B31">
-        <v>471</v>
+        <v>444</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46277.3125</v>
+        <v>46278.3125</v>
       </c>
       <c r="B32">
-        <v>483</v>
+        <v>444</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46277.32291666666</v>
+        <v>46278.32291666666</v>
       </c>
       <c r="B33">
-        <v>483</v>
+        <v>446</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46277.33333333334</v>
+        <v>46278.33333333334</v>
       </c>
       <c r="B34">
-        <v>516</v>
+        <v>445</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46277.34375</v>
+        <v>46278.34375</v>
       </c>
       <c r="B35">
-        <v>657</v>
+        <v>435</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46277.35416666666</v>
+        <v>46278.35416666666</v>
       </c>
       <c r="B36">
-        <v>656</v>
+        <v>433</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46277.36458333334</v>
+        <v>46278.36458333334</v>
       </c>
       <c r="B37">
-        <v>652</v>
+        <v>433</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46277.375</v>
+        <v>46278.375</v>
       </c>
       <c r="B38">
-        <v>381</v>
+        <v>243</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46277.38541666666</v>
+        <v>46278.38541666666</v>
       </c>
       <c r="B39">
-        <v>357</v>
+        <v>226</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46277.39583333334</v>
+        <v>46278.39583333334</v>
       </c>
       <c r="B40">
-        <v>370</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46277.40625</v>
+        <v>46278.40625</v>
       </c>
       <c r="B41">
-        <v>324</v>
+        <v>227</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46277.41666666666</v>
+        <v>46278.41666666666</v>
       </c>
       <c r="B42">
-        <v>327</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46277.42708333334</v>
+        <v>46278.42708333334</v>
       </c>
       <c r="B43">
-        <v>303</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46277.4375</v>
+        <v>46278.4375</v>
       </c>
       <c r="B44">
-        <v>297</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46277.44791666666</v>
+        <v>46278.44791666666</v>
       </c>
       <c r="B45">
-        <v>314</v>
+        <v>201</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46277.45833333334</v>
+        <v>46278.45833333334</v>
       </c>
       <c r="B46">
-        <v>402</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46277.46875</v>
+        <v>46278.46875</v>
       </c>
       <c r="B47">
-        <v>400</v>
+        <v>197</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46277.47916666666</v>
+        <v>46278.47916666666</v>
       </c>
       <c r="B48">
-        <v>364</v>
+        <v>198</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46277.48958333334</v>
+        <v>46278.48958333334</v>
       </c>
       <c r="B49">
-        <v>439</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46277.5</v>
+        <v>46278.5</v>
       </c>
       <c r="B50">
-        <v>332</v>
+        <v>204</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46277.51041666666</v>
+        <v>46278.51041666666</v>
       </c>
       <c r="B51">
-        <v>332</v>
+        <v>205</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46277.52083333334</v>
+        <v>46278.52083333334</v>
       </c>
       <c r="B52">
-        <v>332</v>
+        <v>204</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46277.53125</v>
+        <v>46278.53125</v>
       </c>
       <c r="B53">
-        <v>333</v>
+        <v>203</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46277.54166666666</v>
+        <v>46278.54166666666</v>
       </c>
       <c r="B54">
-        <v>270</v>
+        <v>210</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46277.55208333334</v>
+        <v>46278.55208333334</v>
       </c>
       <c r="B55">
-        <v>265</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46277.5625</v>
+        <v>46278.5625</v>
       </c>
       <c r="B56">
-        <v>264</v>
+        <v>210</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46277.57291666666</v>
+        <v>46278.57291666666</v>
       </c>
       <c r="B57">
-        <v>265</v>
+        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46277.58333333334</v>
+        <v>46278.58333333334</v>
       </c>
       <c r="B58">
-        <v>279</v>
+        <v>201</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46277.59375</v>
+        <v>46278.59375</v>
       </c>
       <c r="B59">
-        <v>280</v>
+        <v>200</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46277.60416666666</v>
+        <v>46278.60416666666</v>
       </c>
       <c r="B60">
-        <v>281</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46277.61458333334</v>
+        <v>46278.61458333334</v>
       </c>
       <c r="B61">
-        <v>282</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46277.625</v>
+        <v>46278.625</v>
       </c>
       <c r="B62">
-        <v>293</v>
+        <v>202</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46277.63541666666</v>
+        <v>46278.63541666666</v>
       </c>
       <c r="B63">
-        <v>295</v>
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46277.64583333334</v>
+        <v>46278.64583333334</v>
       </c>
       <c r="B64">
-        <v>296</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46277.65625</v>
+        <v>46278.65625</v>
       </c>
       <c r="B65">
-        <v>301</v>
+        <v>174</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46277.66666666666</v>
+        <v>46278.66666666666</v>
       </c>
       <c r="B66">
-        <v>441</v>
+        <v>271</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46277.67708333334</v>
+        <v>46278.67708333334</v>
       </c>
       <c r="B67">
-        <v>449</v>
+        <v>291</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46277.6875</v>
+        <v>46278.6875</v>
       </c>
       <c r="B68">
-        <v>450</v>
+        <v>292</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46277.69791666666</v>
+        <v>46278.69791666666</v>
       </c>
       <c r="B69">
-        <v>456</v>
+        <v>311</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46277.70833333334</v>
+        <v>46278.70833333334</v>
       </c>
       <c r="B70">
-        <v>627</v>
+        <v>615</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46277.71875</v>
+        <v>46278.71875</v>
       </c>
       <c r="B71">
-        <v>628</v>
+        <v>638</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46277.72916666666</v>
+        <v>46278.72916666666</v>
       </c>
       <c r="B72">
-        <v>620</v>
+        <v>645</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46277.73958333334</v>
+        <v>46278.73958333334</v>
       </c>
       <c r="B73">
-        <v>615</v>
+        <v>644</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46277.75</v>
+        <v>46278.75</v>
       </c>
       <c r="B74">
-        <v>601</v>
+        <v>628</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46277.76041666666</v>
+        <v>46278.76041666666</v>
       </c>
       <c r="B75">
-        <v>600</v>
+        <v>641</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46277.77083333334</v>
+        <v>46278.77083333334</v>
       </c>
       <c r="B76">
-        <v>603</v>
+        <v>642</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46277.78125</v>
+        <v>46278.78125</v>
       </c>
       <c r="B77">
-        <v>610</v>
+        <v>663</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46277.79166666666</v>
+        <v>46278.79166666666</v>
       </c>
       <c r="B78">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46277.80208333334</v>
+        <v>46278.80208333334</v>
       </c>
       <c r="B79">
-        <v>631</v>
+        <v>621</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46277.8125</v>
+        <v>46278.8125</v>
       </c>
       <c r="B80">
-        <v>705</v>
+        <v>643</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46277.82291666666</v>
+        <v>46278.82291666666</v>
       </c>
       <c r="B81">
-        <v>708</v>
+        <v>643</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46277.83333333334</v>
+        <v>46278.83333333334</v>
       </c>
       <c r="B82">
-        <v>615</v>
+        <v>630</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46277.84375</v>
+        <v>46278.84375</v>
       </c>
       <c r="B83">
-        <v>612</v>
+        <v>628</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46277.85416666666</v>
+        <v>46278.85416666666</v>
       </c>
       <c r="B84">
-        <v>610</v>
+        <v>628</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46277.86458333334</v>
+        <v>46278.86458333334</v>
       </c>
       <c r="B85">
-        <v>610</v>
+        <v>627</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46277.875</v>
+        <v>46278.875</v>
       </c>
       <c r="B86">
-        <v>617</v>
+        <v>625</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46277.88541666666</v>
+        <v>46278.88541666666</v>
       </c>
       <c r="B87">
-        <v>617</v>
+        <v>636</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46277.89583333334</v>
+        <v>46278.89583333334</v>
       </c>
       <c r="B88">
-        <v>589</v>
+        <v>654</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46277.90625</v>
+        <v>46278.90625</v>
       </c>
       <c r="B89">
-        <v>589</v>
+        <v>656</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46277.91666666666</v>
+        <v>46278.91666666666</v>
       </c>
       <c r="B90">
-        <v>577</v>
+        <v>668</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46277.92708333334</v>
+        <v>46278.92708333334</v>
       </c>
       <c r="B91">
-        <v>578</v>
+        <v>668</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46277.9375</v>
+        <v>46278.9375</v>
       </c>
       <c r="B92">
-        <v>578</v>
+        <v>667</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46277.94791666666</v>
+        <v>46278.94791666666</v>
       </c>
       <c r="B93">
-        <v>578</v>
+        <v>667</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46277.95833333334</v>
+        <v>46278.95833333334</v>
       </c>
       <c r="B94">
-        <v>463</v>
+        <v>553</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46277.96875</v>
+        <v>46278.96875</v>
       </c>
       <c r="B95">
-        <v>447</v>
+        <v>535</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46277.97916666666</v>
+        <v>46278.97916666666</v>
       </c>
       <c r="B96">
-        <v>447</v>
+        <v>530</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46277.98958333334</v>
+        <v>46278.98958333334</v>
       </c>
       <c r="B97">
-        <v>448</v>
+        <v>523</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B98">
-        <v>428</v>
+        <v>381</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46278.01041666666</v>
+        <v>46279.01041666666</v>
       </c>
       <c r="B99">
-        <v>427</v>
+        <v>380</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46278.02083333334</v>
+        <v>46279.02083333334</v>
       </c>
       <c r="B100">
-        <v>428</v>
+        <v>380</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46278.03125</v>
+        <v>46279.03125</v>
       </c>
       <c r="B101">
-        <v>427</v>
+        <v>379</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46278.04166666666</v>
+        <v>46279.04166666666</v>
       </c>
       <c r="B102">
-        <v>423</v>
+        <v>380</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46278.05208333334</v>
+        <v>46279.05208333334</v>
       </c>
       <c r="B103">
-        <v>411</v>
+        <v>377</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46278.0625</v>
+        <v>46279.0625</v>
       </c>
       <c r="B104">
-        <v>403</v>
+        <v>380</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46278.07291666666</v>
+        <v>46279.07291666666</v>
       </c>
       <c r="B105">
-        <v>402</v>
+        <v>380</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46278.08333333334</v>
+        <v>46279.08333333334</v>
       </c>
       <c r="B106">
-        <v>415</v>
+        <v>382</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46278.09375</v>
+        <v>46279.09375</v>
       </c>
       <c r="B107">
-        <v>417</v>
+        <v>387</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46278.10416666666</v>
+        <v>46279.10416666666</v>
       </c>
       <c r="B108">
-        <v>416</v>
+        <v>442</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46278.11458333334</v>
+        <v>46279.11458333334</v>
       </c>
       <c r="B109">
-        <v>418</v>
+        <v>445</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46278.125</v>
+        <v>46279.125</v>
       </c>
       <c r="B110">
-        <v>340</v>
+        <v>449</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46278.13541666666</v>
+        <v>46279.13541666666</v>
       </c>
       <c r="B111">
-        <v>336</v>
+        <v>398</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46278.14583333334</v>
+        <v>46279.14583333334</v>
       </c>
       <c r="B112">
-        <v>335</v>
+        <v>389</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46278.15625</v>
+        <v>46279.15625</v>
       </c>
       <c r="B113">
-        <v>336</v>
+        <v>390</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46278.16666666666</v>
+        <v>46279.16666666666</v>
       </c>
       <c r="B114">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46278.17708333334</v>
+        <v>46279.17708333334</v>
       </c>
       <c r="B115">
-        <v>399</v>
+        <v>390</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46278.1875</v>
+        <v>46279.1875</v>
       </c>
       <c r="B116">
-        <v>400</v>
+        <v>390</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46278.19791666666</v>
+        <v>46279.19791666666</v>
       </c>
       <c r="B117">
-        <v>401</v>
+        <v>391</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46278.20833333334</v>
+        <v>46279.20833333334</v>
       </c>
       <c r="B118">
-        <v>441</v>
+        <v>424</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46278.21875</v>
+        <v>46279.21875</v>
       </c>
       <c r="B119">
-        <v>441</v>
+        <v>425</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46278.22916666666</v>
+        <v>46279.22916666666</v>
       </c>
       <c r="B120">
-        <v>433</v>
+        <v>425</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46278.23958333334</v>
+        <v>46279.23958333334</v>
       </c>
       <c r="B121">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46278.25</v>
+        <v>46279.25</v>
       </c>
       <c r="B122">
-        <v>447</v>
+        <v>435</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46278.26041666666</v>
+        <v>46279.26041666666</v>
       </c>
       <c r="B123">
-        <v>451</v>
+        <v>434</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46278.27083333334</v>
+        <v>46279.27083333334</v>
       </c>
       <c r="B124">
-        <v>452</v>
+        <v>435</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46278.28125</v>
+        <v>46279.28125</v>
       </c>
       <c r="B125">
-        <v>453</v>
+        <v>434</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46278.29166666666</v>
+        <v>46279.29166666666</v>
       </c>
       <c r="B126">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46278.30208333334</v>
+        <v>46279.30208333334</v>
       </c>
       <c r="B127">
-        <v>444</v>
+        <v>462</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46278.3125</v>
+        <v>46279.3125</v>
       </c>
       <c r="B128">
-        <v>444</v>
+        <v>463</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46278.32291666666</v>
+        <v>46279.32291666666</v>
       </c>
       <c r="B129">
-        <v>446</v>
+        <v>464</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46278.33333333334</v>
+        <v>46279.33333333334</v>
       </c>
       <c r="B130">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46278.34375</v>
+        <v>46279.34375</v>
       </c>
       <c r="B131">
-        <v>435</v>
+        <v>439</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="2">
+        <v>46279.35416666666</v>
+      </c>
+      <c r="B132">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="2">
+        <v>46279.36458333334</v>
+      </c>
+      <c r="B133">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="2">
+        <v>46279.375</v>
+      </c>
+      <c r="B134">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="2">
+        <v>46279.38541666666</v>
+      </c>
+      <c r="B135">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="2">
+        <v>46279.39583333334</v>
+      </c>
+      <c r="B136">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="2">
+        <v>46279.40625</v>
+      </c>
+      <c r="B137">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="2">
+        <v>46279.41666666666</v>
+      </c>
+      <c r="B138">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="2">
+        <v>46279.42708333334</v>
+      </c>
+      <c r="B139">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="2">
+        <v>46279.4375</v>
+      </c>
+      <c r="B140">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="2">
+        <v>46279.44791666666</v>
+      </c>
+      <c r="B141">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="2">
+        <v>46279.45833333334</v>
+      </c>
+      <c r="B142">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="2">
+        <v>46279.46875</v>
+      </c>
+      <c r="B143">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="2">
+        <v>46279.47916666666</v>
+      </c>
+      <c r="B144">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="2">
+        <v>46279.48958333334</v>
+      </c>
+      <c r="B145">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="2">
+        <v>46279.5</v>
+      </c>
+      <c r="B146">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="2">
+        <v>46279.51041666666</v>
+      </c>
+      <c r="B147">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="2">
+        <v>46279.52083333334</v>
+      </c>
+      <c r="B148">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="2">
+        <v>46279.53125</v>
+      </c>
+      <c r="B149">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="2">
+        <v>46279.54166666666</v>
+      </c>
+      <c r="B150">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46279.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46279.5625</v>
+      </c>
+      <c r="B152">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46279.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46279.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46279.59375</v>
+      </c>
+      <c r="B155">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="2">
+        <v>46279.60416666666</v>
+      </c>
+      <c r="B156">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="2">
+        <v>46279.61458333334</v>
+      </c>
+      <c r="B157">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="2">
+        <v>46279.625</v>
+      </c>
+      <c r="B158">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="2">
+        <v>46279.63541666666</v>
+      </c>
+      <c r="B159">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="2">
+        <v>46279.64583333334</v>
+      </c>
+      <c r="B160">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="2">
+        <v>46279.65625</v>
+      </c>
+      <c r="B161">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="2">
+        <v>46279.66666666666</v>
+      </c>
+      <c r="B162">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2">
+        <v>46279.67708333334</v>
+      </c>
+      <c r="B163">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="2">
+        <v>46279.6875</v>
+      </c>
+      <c r="B164">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2">
+        <v>46279.69791666666</v>
+      </c>
+      <c r="B165">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2">
+        <v>46279.70833333334</v>
+      </c>
+      <c r="B166">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="2">
+        <v>46279.71875</v>
+      </c>
+      <c r="B167">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="2">
+        <v>46279.72916666666</v>
+      </c>
+      <c r="B168">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="2">
+        <v>46279.73958333334</v>
+      </c>
+      <c r="B169">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="2">
+        <v>46279.75</v>
+      </c>
+      <c r="B170">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="2">
+        <v>46279.76041666666</v>
+      </c>
+      <c r="B171">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="2">
+        <v>46279.77083333334</v>
+      </c>
+      <c r="B172">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46279.78125</v>
+      </c>
+      <c r="B173">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46279.79166666666</v>
+      </c>
+      <c r="B174">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46279.80208333334</v>
+      </c>
+      <c r="B175">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46279.8125</v>
+      </c>
+      <c r="B176">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46279.82291666666</v>
+      </c>
+      <c r="B177">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46279.83333333334</v>
+      </c>
+      <c r="B178">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="2">
+        <v>46279.84375</v>
+      </c>
+      <c r="B179">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="2">
+        <v>46279.85416666666</v>
+      </c>
+      <c r="B180">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="2">
+        <v>46279.86458333334</v>
+      </c>
+      <c r="B181">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="2">
+        <v>46279.875</v>
+      </c>
+      <c r="B182">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="2">
+        <v>46279.88541666666</v>
+      </c>
+      <c r="B183">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="2">
+        <v>46279.89583333334</v>
+      </c>
+      <c r="B184">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2">
+        <v>46279.90625</v>
+      </c>
+      <c r="B185">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="2">
+        <v>46279.91666666666</v>
+      </c>
+      <c r="B186">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="2">
+        <v>46279.92708333334</v>
+      </c>
+      <c r="B187">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2">
+        <v>46279.9375</v>
+      </c>
+      <c r="B188">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="2">
+        <v>46279.94791666666</v>
+      </c>
+      <c r="B189">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2">
+        <v>46279.95833333334</v>
+      </c>
+      <c r="B190">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2">
+        <v>46279.96875</v>
+      </c>
+      <c r="B191">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="2">
+        <v>46279.97916666666</v>
+      </c>
+      <c r="B192">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2">
+        <v>46279.98958333334</v>
+      </c>
+      <c r="B193">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46280</v>
+      </c>
+      <c r="B194">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46280.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46280.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46280.03125</v>
+      </c>
+      <c r="B197">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46280.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46280.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46280.0625</v>
+      </c>
+      <c r="B200">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46280.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46280.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46280.09375</v>
+      </c>
+      <c r="B203">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46280.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46280.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46280.125</v>
+      </c>
+      <c r="B206">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46280.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46280.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46280.15625</v>
+      </c>
+      <c r="B209">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46280.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46280.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46280.1875</v>
+      </c>
+      <c r="B212">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46280.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46280.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46280.21875</v>
+      </c>
+      <c r="B215">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46280.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46280.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46280.25</v>
+      </c>
+      <c r="B218">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46280.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46280.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46280.28125</v>
+      </c>
+      <c r="B221">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46280.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46280.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46280.3125</v>
+      </c>
+      <c r="B224">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46280.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46280.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46280.34375</v>
+      </c>
+      <c r="B227">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46280.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46280.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46280.375</v>
+      </c>
+      <c r="B230">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46280.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46280.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46280.40625</v>
+      </c>
+      <c r="B233">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46280.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46280.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46280.4375</v>
+      </c>
+      <c r="B236">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46280.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46280.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46280.46875</v>
+      </c>
+      <c r="B239">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46280.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46280.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46280.5</v>
+      </c>
+      <c r="B242">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46280.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46280.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46280.53125</v>
+      </c>
+      <c r="B245">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46280.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46280.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46280.5625</v>
+      </c>
+      <c r="B248">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46280.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46280.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46280.59375</v>
+      </c>
+      <c r="B251">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46280.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46280.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46280.625</v>
+      </c>
+      <c r="B254">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46280.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46280.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46280.65625</v>
+      </c>
+      <c r="B257">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46280.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46280.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46280.6875</v>
+      </c>
+      <c r="B260">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46280.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46280.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46280.71875</v>
+      </c>
+      <c r="B263">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46280.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46280.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46280.75</v>
+      </c>
+      <c r="B266">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46280.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46280.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46280.78125</v>
+      </c>
+      <c r="B269">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46280.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46280.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46280.8125</v>
+      </c>
+      <c r="B272">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46280.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46280.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46280.84375</v>
+      </c>
+      <c r="B275">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46280.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46280.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46280.875</v>
+      </c>
+      <c r="B278">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46280.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46280.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46280.90625</v>
+      </c>
+      <c r="B281">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46280.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46280.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46280.9375</v>
+      </c>
+      <c r="B284">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46280.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46280.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46280.96875</v>
+      </c>
+      <c r="B287">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46280.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46280.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46281</v>
+      </c>
+      <c r="B290">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46281.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46281.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46281.03125</v>
+      </c>
+      <c r="B293">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46281.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46281.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46281.0625</v>
+      </c>
+      <c r="B296">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46281.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46281.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46281.09375</v>
+      </c>
+      <c r="B299">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46281.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46281.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46281.125</v>
+      </c>
+      <c r="B302">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46281.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46281.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46281.15625</v>
+      </c>
+      <c r="B305">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46281.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46281.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46281.1875</v>
+      </c>
+      <c r="B308">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46281.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46281.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46281.21875</v>
+      </c>
+      <c r="B311">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46281.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46281.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46281.25</v>
+      </c>
+      <c r="B314">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46281.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46281.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46281.28125</v>
+      </c>
+      <c r="B317">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46281.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46281.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46281.3125</v>
+      </c>
+      <c r="B320">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46281.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46281.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46281.34375</v>
+      </c>
+      <c r="B323">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46281.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46281.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46281.375</v>
+      </c>
+      <c r="B326">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46281.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2">
+        <v>46281.39583333334</v>
+      </c>
+      <c r="B328">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="2">
+        <v>46281.40625</v>
+      </c>
+      <c r="B329">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="2">
+        <v>46281.41666666666</v>
+      </c>
+      <c r="B330">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2">
+      <c r="A331" s="2">
+        <v>46281.42708333334</v>
+      </c>
+      <c r="B331">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2">
+      <c r="A332" s="2">
+        <v>46281.4375</v>
+      </c>
+      <c r="B332">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2">
+      <c r="A333" s="2">
+        <v>46281.44791666666</v>
+      </c>
+      <c r="B333">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2">
+      <c r="A334" s="2">
+        <v>46281.45833333334</v>
+      </c>
+      <c r="B334">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2">
+      <c r="A335" s="2">
+        <v>46281.46875</v>
+      </c>
+      <c r="B335">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2">
+      <c r="A336" s="2">
+        <v>46281.47916666666</v>
+      </c>
+      <c r="B336">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" s="2">
+        <v>46281.48958333334</v>
+      </c>
+      <c r="B337">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" s="2">
+        <v>46281.5</v>
+      </c>
+      <c r="B338">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" s="2">
+        <v>46281.51041666666</v>
+      </c>
+      <c r="B339">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" s="2">
+        <v>46281.52083333334</v>
+      </c>
+      <c r="B340">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="A341" s="2">
+        <v>46281.53125</v>
+      </c>
+      <c r="B341">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2">
+      <c r="A342" s="2">
+        <v>46281.54166666666</v>
+      </c>
+      <c r="B342">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="A343" s="2">
+        <v>46281.55208333334</v>
+      </c>
+      <c r="B343">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" s="2">
+        <v>46281.5625</v>
+      </c>
+      <c r="B344">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2">
+      <c r="A345" s="2">
+        <v>46281.57291666666</v>
+      </c>
+      <c r="B345">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="A346" s="2">
+        <v>46281.58333333334</v>
+      </c>
+      <c r="B346">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="A347" s="2">
+        <v>46281.59375</v>
+      </c>
+      <c r="B347">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2">
+      <c r="A348" s="2">
+        <v>46281.60416666666</v>
+      </c>
+      <c r="B348">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" s="2">
+        <v>46281.61458333334</v>
+      </c>
+      <c r="B349">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="A350" s="2">
+        <v>46281.625</v>
+      </c>
+      <c r="B350">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2">
+      <c r="A351" s="2">
+        <v>46281.63541666666</v>
+      </c>
+      <c r="B351">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" s="2">
+        <v>46281.64583333334</v>
+      </c>
+      <c r="B352">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2">
+      <c r="A353" s="2">
+        <v>46281.65625</v>
+      </c>
+      <c r="B353">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2">
+      <c r="A354" s="2">
+        <v>46281.66666666666</v>
+      </c>
+      <c r="B354">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="A355" s="2">
+        <v>46281.67708333334</v>
+      </c>
+      <c r="B355">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2">
+      <c r="A356" s="2">
+        <v>46281.6875</v>
+      </c>
+      <c r="B356">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" s="2">
+        <v>46281.69791666666</v>
+      </c>
+      <c r="B357">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" s="2">
+        <v>46281.70833333334</v>
+      </c>
+      <c r="B358">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" s="2">
+        <v>46281.71875</v>
+      </c>
+      <c r="B359">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" s="2">
+        <v>46281.72916666666</v>
+      </c>
+      <c r="B360">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2">
+      <c r="A361" s="2">
+        <v>46281.73958333334</v>
+      </c>
+      <c r="B361">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" s="2">
+        <v>46281.75</v>
+      </c>
+      <c r="B362">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" s="2">
+        <v>46281.76041666666</v>
+      </c>
+      <c r="B363">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" s="2">
+        <v>46281.77083333334</v>
+      </c>
+      <c r="B364">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2">
+      <c r="A365" s="2">
+        <v>46281.78125</v>
+      </c>
+      <c r="B365">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" s="2">
+        <v>46281.79166666666</v>
+      </c>
+      <c r="B366">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" s="2">
+        <v>46281.80208333334</v>
+      </c>
+      <c r="B367">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" s="2">
+        <v>46281.8125</v>
+      </c>
+      <c r="B368">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" s="2">
+        <v>46281.82291666666</v>
+      </c>
+      <c r="B369">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" s="2">
+        <v>46281.83333333334</v>
+      </c>
+      <c r="B370">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" s="2">
+        <v>46281.84375</v>
+      </c>
+      <c r="B371">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" s="2">
+        <v>46281.85416666666</v>
+      </c>
+      <c r="B372">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" s="2">
+        <v>46281.86458333334</v>
+      </c>
+      <c r="B373">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" s="2">
+        <v>46281.875</v>
+      </c>
+      <c r="B374">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" s="2">
+        <v>46281.88541666666</v>
+      </c>
+      <c r="B375">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" s="2">
+        <v>46281.89583333334</v>
+      </c>
+      <c r="B376">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" s="2">
+        <v>46281.90625</v>
+      </c>
+      <c r="B377">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" s="2">
+        <v>46281.91666666666</v>
+      </c>
+      <c r="B378">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2">
+      <c r="A379" s="2">
+        <v>46281.92708333334</v>
+      </c>
+      <c r="B379">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" s="2">
+        <v>46281.9375</v>
+      </c>
+      <c r="B380">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" s="2">
+        <v>46281.94791666666</v>
+      </c>
+      <c r="B381">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" s="2">
+        <v>46281.95833333334</v>
+      </c>
+      <c r="B382">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" s="2">
+        <v>46281.96875</v>
+      </c>
+      <c r="B383">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" s="2">
+        <v>46281.97916666666</v>
+      </c>
+      <c r="B384">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" s="2">
+        <v>46281.98958333334</v>
+      </c>
+      <c r="B385">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" s="2">
+        <v>46282</v>
+      </c>
+      <c r="B386">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2">
+      <c r="A387" s="2">
+        <v>46282.01041666666</v>
+      </c>
+      <c r="B387">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2">
+      <c r="A388" s="2">
+        <v>46282.02083333334</v>
+      </c>
+      <c r="B388">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" s="2">
+        <v>46282.03125</v>
+      </c>
+      <c r="B389">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2">
+      <c r="A390" s="2">
+        <v>46282.04166666666</v>
+      </c>
+      <c r="B390">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" s="2">
+        <v>46282.05208333334</v>
+      </c>
+      <c r="B391">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" s="2">
+        <v>46282.0625</v>
+      </c>
+      <c r="B392">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2">
+      <c r="A393" s="2">
+        <v>46282.07291666666</v>
+      </c>
+      <c r="B393">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2">
+      <c r="A394" s="2">
+        <v>46282.08333333334</v>
+      </c>
+      <c r="B394">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2">
+      <c r="A395" s="2">
+        <v>46282.09375</v>
+      </c>
+      <c r="B395">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2">
+      <c r="A396" s="2">
+        <v>46282.10416666666</v>
+      </c>
+      <c r="B396">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2">
+      <c r="A397" s="2">
+        <v>46282.11458333334</v>
+      </c>
+      <c r="B397">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2">
+      <c r="A398" s="2">
+        <v>46282.125</v>
+      </c>
+      <c r="B398">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2">
+      <c r="A399" s="2">
+        <v>46282.13541666666</v>
+      </c>
+      <c r="B399">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2">
+      <c r="A400" s="2">
+        <v>46282.14583333334</v>
+      </c>
+      <c r="B400">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2">
+      <c r="A401" s="2">
+        <v>46282.15625</v>
+      </c>
+      <c r="B401">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2">
+      <c r="A402" s="2">
+        <v>46282.16666666666</v>
+      </c>
+      <c r="B402">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2">
+      <c r="A403" s="2">
+        <v>46282.17708333334</v>
+      </c>
+      <c r="B403">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2">
+      <c r="A404" s="2">
+        <v>46282.1875</v>
+      </c>
+      <c r="B404">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" s="2">
+        <v>46282.19791666666</v>
+      </c>
+      <c r="B405">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2">
+      <c r="A406" s="2">
+        <v>46282.20833333334</v>
+      </c>
+      <c r="B406">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2">
+      <c r="A407" s="2">
+        <v>46282.21875</v>
+      </c>
+      <c r="B407">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" s="2">
+        <v>46282.22916666666</v>
+      </c>
+      <c r="B408">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2">
+      <c r="A409" s="2">
+        <v>46282.23958333334</v>
+      </c>
+      <c r="B409">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2">
+      <c r="A410" s="2">
+        <v>46282.25</v>
+      </c>
+      <c r="B410">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2">
+      <c r="A411" s="2">
+        <v>46282.26041666666</v>
+      </c>
+      <c r="B411">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2">
+      <c r="A412" s="2">
+        <v>46282.27083333334</v>
+      </c>
+      <c r="B412">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2">
+      <c r="A413" s="2">
+        <v>46282.28125</v>
+      </c>
+      <c r="B413">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2">
+      <c r="A414" s="2">
+        <v>46282.29166666666</v>
+      </c>
+      <c r="B414">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2">
+      <c r="A415" s="2">
+        <v>46282.30208333334</v>
+      </c>
+      <c r="B415">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2">
+      <c r="A416" s="2">
+        <v>46282.3125</v>
+      </c>
+      <c r="B416">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2">
+      <c r="A417" s="2">
+        <v>46282.32291666666</v>
+      </c>
+      <c r="B417">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2">
+      <c r="A418" s="2">
+        <v>46282.33333333334</v>
+      </c>
+      <c r="B418">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2">
+      <c r="A419" s="2">
+        <v>46282.34375</v>
+      </c>
+      <c r="B419">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="420" spans="1:2">
+      <c r="A420" s="2">
+        <v>46282.35416666666</v>
+      </c>
+      <c r="B420">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="421" spans="1:2">
+      <c r="A421" s="2">
+        <v>46282.36458333334</v>
+      </c>
+      <c r="B421">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2">
+      <c r="A422" s="2">
+        <v>46282.375</v>
+      </c>
+      <c r="B422">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2">
+      <c r="A423" s="2">
+        <v>46282.38541666666</v>
+      </c>
+      <c r="B423">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2">
+      <c r="A424" s="2">
+        <v>46282.39583333334</v>
+      </c>
+      <c r="B424">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2">
+      <c r="A425" s="2">
+        <v>46282.40625</v>
+      </c>
+      <c r="B425">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2">
+      <c r="A426" s="2">
+        <v>46282.41666666666</v>
+      </c>
+      <c r="B426">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2">
+      <c r="A427" s="2">
+        <v>46282.42708333334</v>
+      </c>
+      <c r="B427">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2">
+      <c r="A428" s="2">
+        <v>46282.4375</v>
+      </c>
+      <c r="B428">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2">
+      <c r="A429" s="2">
+        <v>46282.44791666666</v>
+      </c>
+      <c r="B429">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" s="2">
+        <v>46282.45833333334</v>
+      </c>
+      <c r="B430">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="431" spans="1:2">
+      <c r="A431" s="2">
+        <v>46282.46875</v>
+      </c>
+      <c r="B431">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2">
+      <c r="A432" s="2">
+        <v>46282.47916666666</v>
+      </c>
+      <c r="B432">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="433" spans="1:2">
+      <c r="A433" s="2">
+        <v>46282.48958333334</v>
+      </c>
+      <c r="B433">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" s="2">
+        <v>46282.5</v>
+      </c>
+      <c r="B434">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2">
+      <c r="A435" s="2">
+        <v>46282.51041666666</v>
+      </c>
+      <c r="B435">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="436" spans="1:2">
+      <c r="A436" s="2">
+        <v>46282.52083333334</v>
+      </c>
+      <c r="B436">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2">
+      <c r="A437" s="2">
+        <v>46282.53125</v>
+      </c>
+      <c r="B437">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2">
+      <c r="A438" s="2">
+        <v>46282.54166666666</v>
+      </c>
+      <c r="B438">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" s="2">
+        <v>46282.55208333334</v>
+      </c>
+      <c r="B439">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" s="2">
+        <v>46282.5625</v>
+      </c>
+      <c r="B440">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2">
+      <c r="A441" s="2">
+        <v>46282.57291666666</v>
+      </c>
+      <c r="B441">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2">
+      <c r="A442" s="2">
+        <v>46282.58333333334</v>
+      </c>
+      <c r="B442">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2">
+      <c r="A443" s="2">
+        <v>46282.59375</v>
+      </c>
+      <c r="B443">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" s="2">
+        <v>46282.60416666666</v>
+      </c>
+      <c r="B444">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2">
+      <c r="A445" s="2">
+        <v>46282.61458333334</v>
+      </c>
+      <c r="B445">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2">
+      <c r="A446" s="2">
+        <v>46282.625</v>
+      </c>
+      <c r="B446">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" s="2">
+        <v>46282.63541666666</v>
+      </c>
+      <c r="B447">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2">
+      <c r="A448" s="2">
+        <v>46282.64583333334</v>
+      </c>
+      <c r="B448">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2">
+      <c r="A449" s="2">
+        <v>46282.65625</v>
+      </c>
+      <c r="B449">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" s="2">
+        <v>46282.66666666666</v>
+      </c>
+      <c r="B450">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" s="2">
+        <v>46282.67708333334</v>
+      </c>
+      <c r="B451">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2">
+      <c r="A452" s="2">
+        <v>46282.6875</v>
+      </c>
+      <c r="B452">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2">
+      <c r="A453" s="2">
+        <v>46282.69791666666</v>
+      </c>
+      <c r="B453">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2">
+      <c r="A454" s="2">
+        <v>46282.70833333334</v>
+      </c>
+      <c r="B454">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" s="2">
+        <v>46282.71875</v>
+      </c>
+      <c r="B455">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" s="2">
+        <v>46282.72916666666</v>
+      </c>
+      <c r="B456">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" s="2">
+        <v>46282.73958333334</v>
+      </c>
+      <c r="B457">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" s="2">
+        <v>46282.75</v>
+      </c>
+      <c r="B458">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" s="2">
+        <v>46282.76041666666</v>
+      </c>
+      <c r="B459">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2">
+      <c r="A460" s="2">
+        <v>46282.77083333334</v>
+      </c>
+      <c r="B460">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" s="2">
+        <v>46282.78125</v>
+      </c>
+      <c r="B461">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" s="2">
+        <v>46282.79166666666</v>
+      </c>
+      <c r="B462">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" s="2">
+        <v>46282.80208333334</v>
+      </c>
+      <c r="B463">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" s="2">
+        <v>46282.8125</v>
+      </c>
+      <c r="B464">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" s="2">
+        <v>46282.82291666666</v>
+      </c>
+      <c r="B465">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" s="2">
+        <v>46282.83333333334</v>
+      </c>
+      <c r="B466">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2">
+      <c r="A467" s="2">
+        <v>46282.84375</v>
+      </c>
+      <c r="B467">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" s="2">
+        <v>46282.85416666666</v>
+      </c>
+      <c r="B468">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" s="2">
+        <v>46282.86458333334</v>
+      </c>
+      <c r="B469">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" s="2">
+        <v>46282.875</v>
+      </c>
+      <c r="B470">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" s="2">
+        <v>46282.88541666666</v>
+      </c>
+      <c r="B471">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" s="2">
+        <v>46282.89583333334</v>
+      </c>
+      <c r="B472">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" s="2">
+        <v>46282.90625</v>
+      </c>
+      <c r="B473">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" s="2">
+        <v>46282.91666666666</v>
+      </c>
+      <c r="B474">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" s="2">
+        <v>46282.92708333334</v>
+      </c>
+      <c r="B475">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" s="2">
+        <v>46282.9375</v>
+      </c>
+      <c r="B476">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" s="2">
+        <v>46282.94791666666</v>
+      </c>
+      <c r="B477">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="478" spans="1:2">
+      <c r="A478" s="2">
+        <v>46282.95833333334</v>
+      </c>
+      <c r="B478">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2">
+      <c r="A479" s="2">
+        <v>46282.96875</v>
+      </c>
+      <c r="B479">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2">
+      <c r="A480" s="2">
+        <v>46282.97916666666</v>
+      </c>
+      <c r="B480">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" s="2">
+        <v>46282.98958333334</v>
+      </c>
+      <c r="B481">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" s="2">
+        <v>46283</v>
+      </c>
+      <c r="B482">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2">
+      <c r="A483" s="2">
+        <v>46283.01041666666</v>
+      </c>
+      <c r="B483">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="484" spans="1:2">
+      <c r="A484" s="2">
+        <v>46283.02083333334</v>
+      </c>
+      <c r="B484">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="485" spans="1:2">
+      <c r="A485" s="2">
+        <v>46283.03125</v>
+      </c>
+      <c r="B485">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="486" spans="1:2">
+      <c r="A486" s="2">
+        <v>46283.04166666666</v>
+      </c>
+      <c r="B486">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2">
+      <c r="A487" s="2">
+        <v>46283.05208333334</v>
+      </c>
+      <c r="B487">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2">
+      <c r="A488" s="2">
+        <v>46283.0625</v>
+      </c>
+      <c r="B488">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" s="2">
+        <v>46283.07291666666</v>
+      </c>
+      <c r="B489">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2">
+      <c r="A490" s="2">
+        <v>46283.08333333334</v>
+      </c>
+      <c r="B490">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="491" spans="1:2">
+      <c r="A491" s="2">
+        <v>46283.09375</v>
+      </c>
+      <c r="B491">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="492" spans="1:2">
+      <c r="A492" s="2">
+        <v>46283.10416666666</v>
+      </c>
+      <c r="B492">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="493" spans="1:2">
+      <c r="A493" s="2">
+        <v>46283.11458333334</v>
+      </c>
+      <c r="B493">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2">
+      <c r="A494" s="2">
+        <v>46283.125</v>
+      </c>
+      <c r="B494">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="495" spans="1:2">
+      <c r="A495" s="2">
+        <v>46283.13541666666</v>
+      </c>
+      <c r="B495">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2">
+      <c r="A496" s="2">
+        <v>46283.14583333334</v>
+      </c>
+      <c r="B496">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="497" spans="1:2">
+      <c r="A497" s="2">
+        <v>46283.15625</v>
+      </c>
+      <c r="B497">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="498" spans="1:2">
+      <c r="A498" s="2">
+        <v>46283.16666666666</v>
+      </c>
+      <c r="B498">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="499" spans="1:2">
+      <c r="A499" s="2">
+        <v>46283.17708333334</v>
+      </c>
+      <c r="B499">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="500" spans="1:2">
+      <c r="A500" s="2">
+        <v>46283.1875</v>
+      </c>
+      <c r="B500">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="501" spans="1:2">
+      <c r="A501" s="2">
+        <v>46283.19791666666</v>
+      </c>
+      <c r="B501">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="502" spans="1:2">
+      <c r="A502" s="2">
+        <v>46283.20833333334</v>
+      </c>
+      <c r="B502">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="503" spans="1:2">
+      <c r="A503" s="2">
+        <v>46283.21875</v>
+      </c>
+      <c r="B503">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="504" spans="1:2">
+      <c r="A504" s="2">
+        <v>46283.22916666666</v>
+      </c>
+      <c r="B504">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="505" spans="1:2">
+      <c r="A505" s="2">
+        <v>46283.23958333334</v>
+      </c>
+      <c r="B505">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="506" spans="1:2">
+      <c r="A506" s="2">
+        <v>46283.25</v>
+      </c>
+      <c r="B506">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="507" spans="1:2">
+      <c r="A507" s="2">
+        <v>46283.26041666666</v>
+      </c>
+      <c r="B507">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="508" spans="1:2">
+      <c r="A508" s="2">
+        <v>46283.27083333334</v>
+      </c>
+      <c r="B508">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2">
+      <c r="A509" s="2">
+        <v>46283.28125</v>
+      </c>
+      <c r="B509">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="510" spans="1:2">
+      <c r="A510" s="2">
+        <v>46283.29166666666</v>
+      </c>
+      <c r="B510">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="511" spans="1:2">
+      <c r="A511" s="2">
+        <v>46283.30208333334</v>
+      </c>
+      <c r="B511">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="512" spans="1:2">
+      <c r="A512" s="2">
+        <v>46283.3125</v>
+      </c>
+      <c r="B512">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="513" spans="1:2">
+      <c r="A513" s="2">
+        <v>46283.32291666666</v>
+      </c>
+      <c r="B513">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="514" spans="1:2">
+      <c r="A514" s="2">
+        <v>46283.33333333334</v>
+      </c>
+      <c r="B514">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="515" spans="1:2">
+      <c r="A515" s="2">
+        <v>46283.34375</v>
+      </c>
+      <c r="B515">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="516" spans="1:2">
+      <c r="A516" s="2">
+        <v>46283.35416666666</v>
+      </c>
+      <c r="B516">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="517" spans="1:2">
+      <c r="A517" s="2">
+        <v>46283.36458333334</v>
+      </c>
+      <c r="B517">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="518" spans="1:2">
+      <c r="A518" s="2">
+        <v>46283.375</v>
+      </c>
+      <c r="B518">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="519" spans="1:2">
+      <c r="A519" s="2">
+        <v>46283.38541666666</v>
+      </c>
+      <c r="B519">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="520" spans="1:2">
+      <c r="A520" s="2">
+        <v>46283.39583333334</v>
+      </c>
+      <c r="B520">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="521" spans="1:2">
+      <c r="A521" s="2">
+        <v>46283.40625</v>
+      </c>
+      <c r="B521">
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for Elnet
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B230"/>
+  <dimension ref="A1:B232"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,1834 +394,1850 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46283</v>
+        <v>46293</v>
       </c>
       <c r="B2">
-        <v>689</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46283.01041666666</v>
+        <v>46293.01041666666</v>
       </c>
       <c r="B3">
-        <v>690</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46283.02083333334</v>
+        <v>46293.02083333334</v>
       </c>
       <c r="B4">
-        <v>690</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46283.03125</v>
+        <v>46293.03125</v>
       </c>
       <c r="B5">
-        <v>690</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46283.04166666666</v>
+        <v>46293.04166666666</v>
       </c>
       <c r="B6">
-        <v>420</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46283.05208333334</v>
+        <v>46293.05208333334</v>
       </c>
       <c r="B7">
-        <v>385</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46283.0625</v>
+        <v>46293.0625</v>
       </c>
       <c r="B8">
-        <v>385</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46283.07291666666</v>
+        <v>46293.07291666666</v>
       </c>
       <c r="B9">
-        <v>384</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46283.08333333334</v>
+        <v>46293.08333333334</v>
       </c>
       <c r="B10">
-        <v>423</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46283.09375</v>
+        <v>46293.09375</v>
       </c>
       <c r="B11">
-        <v>426</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46283.10416666666</v>
+        <v>46293.10416666666</v>
       </c>
       <c r="B12">
-        <v>424</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46283.11458333334</v>
+        <v>46293.11458333334</v>
       </c>
       <c r="B13">
-        <v>426</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46283.125</v>
+        <v>46293.125</v>
       </c>
       <c r="B14">
-        <v>425</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46283.13541666666</v>
+        <v>46293.13541666666</v>
       </c>
       <c r="B15">
-        <v>426</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46283.14583333334</v>
+        <v>46293.14583333334</v>
       </c>
       <c r="B16">
-        <v>425</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46283.15625</v>
+        <v>46293.15625</v>
       </c>
       <c r="B17">
-        <v>425</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46283.16666666666</v>
+        <v>46293.16666666666</v>
       </c>
       <c r="B18">
-        <v>423</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46283.17708333334</v>
+        <v>46293.17708333334</v>
       </c>
       <c r="B19">
-        <v>424</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46283.1875</v>
+        <v>46293.1875</v>
       </c>
       <c r="B20">
-        <v>423</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46283.19791666666</v>
+        <v>46293.19791666666</v>
       </c>
       <c r="B21">
-        <v>425</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46283.20833333334</v>
+        <v>46293.20833333334</v>
       </c>
       <c r="B22">
-        <v>449</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46283.21875</v>
+        <v>46293.21875</v>
       </c>
       <c r="B23">
-        <v>461</v>
+        <v>313</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46283.22916666666</v>
+        <v>46293.22916666666</v>
       </c>
       <c r="B24">
-        <v>556</v>
+        <v>314</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46283.23958333334</v>
+        <v>46293.23958333334</v>
       </c>
       <c r="B25">
-        <v>551</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46283.25</v>
+        <v>46293.25</v>
       </c>
       <c r="B26">
-        <v>663</v>
+        <v>598</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46283.26041666666</v>
+        <v>46293.26041666666</v>
       </c>
       <c r="B27">
-        <v>667</v>
+        <v>612</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46283.27083333334</v>
+        <v>46293.27083333334</v>
       </c>
       <c r="B28">
-        <v>666</v>
+        <v>606</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46283.28125</v>
+        <v>46293.28125</v>
       </c>
       <c r="B29">
-        <v>666</v>
+        <v>623</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46283.29166666666</v>
+        <v>46293.29166666666</v>
       </c>
       <c r="B30">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46283.30208333334</v>
+        <v>46293.30208333334</v>
       </c>
       <c r="B31">
-        <v>648</v>
+        <v>623</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46283.3125</v>
+        <v>46293.3125</v>
       </c>
       <c r="B32">
-        <v>682</v>
+        <v>627</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46283.32291666666</v>
+        <v>46293.32291666666</v>
       </c>
       <c r="B33">
-        <v>707</v>
+        <v>630</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46283.33333333334</v>
+        <v>46293.33333333334</v>
       </c>
       <c r="B34">
-        <v>567</v>
+        <v>314</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46283.34375</v>
+        <v>46293.34375</v>
       </c>
       <c r="B35">
-        <v>559</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46283.35416666666</v>
+        <v>46293.35416666666</v>
       </c>
       <c r="B36">
-        <v>522</v>
+        <v>231</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46283.36458333334</v>
+        <v>46293.36458333334</v>
       </c>
       <c r="B37">
-        <v>519</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46283.375</v>
+        <v>46293.375</v>
       </c>
       <c r="B38">
-        <v>332</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46283.38541666666</v>
+        <v>46293.38541666666</v>
       </c>
       <c r="B39">
-        <v>306</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46283.39583333334</v>
+        <v>46293.39583333334</v>
       </c>
       <c r="B40">
-        <v>305</v>
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46283.40625</v>
+        <v>46293.40625</v>
       </c>
       <c r="B41">
-        <v>304</v>
+        <v>213</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46283.41666666666</v>
+        <v>46293.41666666666</v>
       </c>
       <c r="B42">
-        <v>265</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46283.42708333334</v>
+        <v>46293.42708333334</v>
       </c>
       <c r="B43">
-        <v>263</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46283.4375</v>
+        <v>46293.4375</v>
       </c>
       <c r="B44">
-        <v>262</v>
+        <v>205</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46283.44791666666</v>
+        <v>46293.44791666666</v>
       </c>
       <c r="B45">
-        <v>262</v>
+        <v>201</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46283.45833333334</v>
+        <v>46293.45833333334</v>
       </c>
       <c r="B46">
-        <v>261</v>
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46283.46875</v>
+        <v>46293.46875</v>
       </c>
       <c r="B47">
-        <v>246</v>
+        <v>185</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46283.47916666666</v>
+        <v>46293.47916666666</v>
       </c>
       <c r="B48">
-        <v>246</v>
+        <v>192</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46283.48958333334</v>
+        <v>46293.48958333334</v>
       </c>
       <c r="B49">
-        <v>245</v>
+        <v>191</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46283.5</v>
+        <v>46293.5</v>
       </c>
       <c r="B50">
-        <v>241</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46283.51041666666</v>
+        <v>46293.51041666666</v>
       </c>
       <c r="B51">
-        <v>240</v>
+        <v>180</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46283.52083333334</v>
+        <v>46293.52083333334</v>
       </c>
       <c r="B52">
-        <v>240</v>
+        <v>216</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46283.53125</v>
+        <v>46293.53125</v>
       </c>
       <c r="B53">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46283.54166666666</v>
+        <v>46293.54166666666</v>
       </c>
       <c r="B54">
-        <v>220</v>
+        <v>181</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46283.55208333334</v>
+        <v>46293.55208333334</v>
       </c>
       <c r="B55">
-        <v>225</v>
+        <v>179</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46283.5625</v>
+        <v>46293.5625</v>
       </c>
       <c r="B56">
-        <v>237</v>
+        <v>180</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46283.57291666666</v>
+        <v>46293.57291666666</v>
       </c>
       <c r="B57">
-        <v>204</v>
+        <v>179</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46283.58333333334</v>
+        <v>46293.58333333334</v>
       </c>
       <c r="B58">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46283.59375</v>
+        <v>46293.59375</v>
       </c>
       <c r="B59">
-        <v>209</v>
+        <v>179</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46283.60416666666</v>
+        <v>46293.60416666666</v>
       </c>
       <c r="B60">
-        <v>239</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46283.61458333334</v>
+        <v>46293.61458333334</v>
       </c>
       <c r="B61">
-        <v>241</v>
+        <v>218</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46283.625</v>
+        <v>46293.625</v>
       </c>
       <c r="B62">
-        <v>246</v>
+        <v>220</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46283.63541666666</v>
+        <v>46293.63541666666</v>
       </c>
       <c r="B63">
-        <v>240</v>
+        <v>221</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46283.64583333334</v>
+        <v>46293.64583333334</v>
       </c>
       <c r="B64">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46283.65625</v>
+        <v>46293.65625</v>
       </c>
       <c r="B65">
-        <v>240</v>
+        <v>221</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46283.66666666666</v>
+        <v>46293.66666666666</v>
       </c>
       <c r="B66">
-        <v>261</v>
+        <v>253</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46283.67708333334</v>
+        <v>46293.67708333334</v>
       </c>
       <c r="B67">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46283.6875</v>
+        <v>46293.6875</v>
       </c>
       <c r="B68">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46283.69791666666</v>
+        <v>46293.69791666666</v>
       </c>
       <c r="B69">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46283.70833333334</v>
+        <v>46293.70833333334</v>
       </c>
       <c r="B70">
-        <v>673</v>
+        <v>735</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46283.71875</v>
+        <v>46293.71875</v>
       </c>
       <c r="B71">
-        <v>695</v>
+        <v>767</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46283.72916666666</v>
+        <v>46293.72916666666</v>
       </c>
       <c r="B72">
-        <v>739</v>
+        <v>764</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46283.73958333334</v>
+        <v>46293.73958333334</v>
       </c>
       <c r="B73">
-        <v>737</v>
+        <v>764</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46283.75</v>
+        <v>46293.75</v>
       </c>
       <c r="B74">
-        <v>743</v>
+        <v>773</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46283.76041666666</v>
+        <v>46293.76041666666</v>
       </c>
       <c r="B75">
-        <v>727</v>
+        <v>776</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46283.77083333334</v>
+        <v>46293.77083333334</v>
       </c>
       <c r="B76">
-        <v>753</v>
+        <v>776</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46283.78125</v>
+        <v>46293.78125</v>
       </c>
       <c r="B77">
-        <v>743</v>
+        <v>779</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46283.79166666666</v>
+        <v>46293.79166666666</v>
       </c>
       <c r="B78">
-        <v>715</v>
+        <v>769</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46283.80208333334</v>
+        <v>46293.80208333334</v>
       </c>
       <c r="B79">
-        <v>713</v>
+        <v>769</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46283.8125</v>
+        <v>46293.8125</v>
       </c>
       <c r="B80">
-        <v>713</v>
+        <v>769</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46283.82291666666</v>
+        <v>46293.82291666666</v>
       </c>
       <c r="B81">
-        <v>715</v>
+        <v>770</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46283.83333333334</v>
+        <v>46293.83333333334</v>
       </c>
       <c r="B82">
-        <v>729</v>
+        <v>761</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46283.84375</v>
+        <v>46293.84375</v>
       </c>
       <c r="B83">
-        <v>730</v>
+        <v>761</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46283.85416666666</v>
+        <v>46293.85416666666</v>
       </c>
       <c r="B84">
-        <v>730</v>
+        <v>762</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46283.86458333334</v>
+        <v>46293.86458333334</v>
       </c>
       <c r="B85">
-        <v>730</v>
+        <v>759</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46283.875</v>
+        <v>46293.875</v>
       </c>
       <c r="B86">
-        <v>719</v>
+        <v>758</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46283.88541666666</v>
+        <v>46293.88541666666</v>
       </c>
       <c r="B87">
-        <v>718</v>
+        <v>757</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46283.89583333334</v>
+        <v>46293.89583333334</v>
       </c>
       <c r="B88">
-        <v>717</v>
+        <v>758</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46283.90625</v>
+        <v>46293.90625</v>
       </c>
       <c r="B89">
-        <v>718</v>
+        <v>752</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46283.91666666666</v>
+        <v>46293.91666666666</v>
       </c>
       <c r="B90">
-        <v>807</v>
+        <v>392</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46283.92708333334</v>
+        <v>46293.92708333334</v>
       </c>
       <c r="B91">
-        <v>812</v>
+        <v>364</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46283.9375</v>
+        <v>46293.9375</v>
       </c>
       <c r="B92">
-        <v>810</v>
+        <v>364</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46283.94791666666</v>
+        <v>46293.94791666666</v>
       </c>
       <c r="B93">
-        <v>808</v>
+        <v>362</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46283.95833333334</v>
+        <v>46293.95833333334</v>
       </c>
       <c r="B94">
-        <v>800</v>
+        <v>301</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46283.96875</v>
+        <v>46293.96875</v>
       </c>
       <c r="B95">
-        <v>810</v>
+        <v>292</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46283.97916666666</v>
+        <v>46293.97916666666</v>
       </c>
       <c r="B96">
-        <v>902</v>
+        <v>304</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46283.98958333334</v>
+        <v>46293.98958333334</v>
       </c>
       <c r="B97">
-        <v>902</v>
+        <v>305</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46284</v>
+        <v>46294</v>
       </c>
       <c r="B98">
-        <v>430</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46284.01041666666</v>
+        <v>46294.01041666666</v>
       </c>
       <c r="B99">
-        <v>383</v>
+        <v>274</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46284.02083333334</v>
+        <v>46294.02083333334</v>
       </c>
       <c r="B100">
-        <v>293</v>
+        <v>274</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46284.03125</v>
+        <v>46294.03125</v>
       </c>
       <c r="B101">
-        <v>289</v>
+        <v>274</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46284.04166666666</v>
+        <v>46294.04166666666</v>
       </c>
       <c r="B102">
-        <v>287</v>
+        <v>265</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46284.05208333334</v>
+        <v>46294.05208333334</v>
       </c>
       <c r="B103">
-        <v>286</v>
+        <v>265</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46284.0625</v>
+        <v>46294.0625</v>
       </c>
       <c r="B104">
-        <v>286</v>
+        <v>265</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46284.07291666666</v>
+        <v>46294.07291666666</v>
       </c>
       <c r="B105">
-        <v>286</v>
+        <v>265</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46284.08333333334</v>
+        <v>46294.08333333334</v>
       </c>
       <c r="B106">
-        <v>278</v>
+        <v>254</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46284.09375</v>
+        <v>46294.09375</v>
       </c>
       <c r="B107">
-        <v>277</v>
+        <v>253</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46284.10416666666</v>
+        <v>46294.10416666666</v>
       </c>
       <c r="B108">
-        <v>277</v>
+        <v>253</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46284.11458333334</v>
+        <v>46294.11458333334</v>
       </c>
       <c r="B109">
-        <v>278</v>
+        <v>253</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46284.125</v>
+        <v>46294.125</v>
       </c>
       <c r="B110">
-        <v>278</v>
+        <v>256</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46284.13541666666</v>
+        <v>46294.13541666666</v>
       </c>
       <c r="B111">
-        <v>278</v>
+        <v>255</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46284.14583333334</v>
+        <v>46294.14583333334</v>
       </c>
       <c r="B112">
-        <v>278</v>
+        <v>256</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46284.15625</v>
+        <v>46294.15625</v>
       </c>
       <c r="B113">
-        <v>281</v>
+        <v>256</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46284.16666666666</v>
+        <v>46294.16666666666</v>
       </c>
       <c r="B114">
-        <v>389</v>
+        <v>283</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46284.17708333334</v>
+        <v>46294.17708333334</v>
       </c>
       <c r="B115">
-        <v>391</v>
+        <v>285</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46284.1875</v>
+        <v>46294.1875</v>
       </c>
       <c r="B116">
-        <v>391</v>
+        <v>284</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46284.19791666666</v>
+        <v>46294.19791666666</v>
       </c>
       <c r="B117">
-        <v>391</v>
+        <v>285</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46284.20833333334</v>
+        <v>46294.20833333334</v>
       </c>
       <c r="B118">
-        <v>419</v>
+        <v>292</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46284.21875</v>
+        <v>46294.21875</v>
       </c>
       <c r="B119">
-        <v>422</v>
+        <v>291</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46284.22916666666</v>
+        <v>46294.22916666666</v>
       </c>
       <c r="B120">
-        <v>413</v>
+        <v>291</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46284.23958333334</v>
+        <v>46294.23958333334</v>
       </c>
       <c r="B121">
-        <v>414</v>
+        <v>306</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46284.25</v>
+        <v>46294.25</v>
       </c>
       <c r="B122">
-        <v>412</v>
+        <v>695</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46284.26041666666</v>
+        <v>46294.26041666666</v>
       </c>
       <c r="B123">
-        <v>409</v>
+        <v>722</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46284.27083333334</v>
+        <v>46294.27083333334</v>
       </c>
       <c r="B124">
-        <v>410</v>
+        <v>722</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46284.28125</v>
+        <v>46294.28125</v>
       </c>
       <c r="B125">
-        <v>409</v>
+        <v>727</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46284.29166666666</v>
+        <v>46294.29166666666</v>
       </c>
       <c r="B126">
-        <v>299</v>
+        <v>722</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46284.30208333334</v>
+        <v>46294.30208333334</v>
       </c>
       <c r="B127">
-        <v>293</v>
+        <v>725</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46284.3125</v>
+        <v>46294.3125</v>
       </c>
       <c r="B128">
-        <v>300</v>
+        <v>727</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46284.32291666666</v>
+        <v>46294.32291666666</v>
       </c>
       <c r="B129">
-        <v>300</v>
+        <v>722</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46284.33333333334</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="B130">
-        <v>275</v>
+        <v>708</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46284.34375</v>
+        <v>46294.34375</v>
       </c>
       <c r="B131">
-        <v>273</v>
+        <v>704</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46284.35416666666</v>
+        <v>46294.35416666666</v>
       </c>
       <c r="B132">
-        <v>273</v>
+        <v>705</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46284.36458333334</v>
+        <v>46294.36458333334</v>
       </c>
       <c r="B133">
-        <v>271</v>
+        <v>705</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46284.375</v>
+        <v>46294.375</v>
       </c>
       <c r="B134">
-        <v>264</v>
+        <v>316</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46284.38541666666</v>
+        <v>46294.38541666666</v>
       </c>
       <c r="B135">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46284.39583333334</v>
+        <v>46294.39583333334</v>
       </c>
       <c r="B136">
-        <v>251</v>
+        <v>262</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46284.40625</v>
+        <v>46294.40625</v>
       </c>
       <c r="B137">
-        <v>251</v>
+        <v>261</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46284.41666666666</v>
+        <v>46294.41666666666</v>
       </c>
       <c r="B138">
-        <v>246</v>
+        <v>258</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46284.42708333334</v>
+        <v>46294.42708333334</v>
       </c>
       <c r="B139">
-        <v>244</v>
+        <v>258</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46284.4375</v>
+        <v>46294.4375</v>
       </c>
       <c r="B140">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46284.44791666666</v>
+        <v>46294.44791666666</v>
       </c>
       <c r="B141">
-        <v>244</v>
+        <v>266</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46284.45833333334</v>
+        <v>46294.45833333334</v>
       </c>
       <c r="B142">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46284.46875</v>
+        <v>46294.46875</v>
       </c>
       <c r="B143">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46284.47916666666</v>
+        <v>46294.47916666666</v>
       </c>
       <c r="B144">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46284.48958333334</v>
+        <v>46294.48958333334</v>
       </c>
       <c r="B145">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46284.5</v>
+        <v>46294.5</v>
       </c>
       <c r="B146">
-        <v>240</v>
+        <v>213</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46284.51041666666</v>
+        <v>46294.51041666666</v>
       </c>
       <c r="B147">
-        <v>240</v>
+        <v>200</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46284.52083333334</v>
+        <v>46294.52083333334</v>
       </c>
       <c r="B148">
-        <v>240</v>
+        <v>201</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46284.53125</v>
+        <v>46294.53125</v>
       </c>
       <c r="B149">
-        <v>240</v>
+        <v>201</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46284.54166666666</v>
+        <v>46294.54166666666</v>
       </c>
       <c r="B150">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="2">
-        <v>46284.55208333334</v>
+        <v>46294.55208333334</v>
       </c>
       <c r="B151">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="2">
-        <v>46284.5625</v>
+        <v>46294.5625</v>
       </c>
       <c r="B152">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153" s="2">
-        <v>46284.57291666666</v>
+        <v>46294.57291666666</v>
       </c>
       <c r="B153">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="2">
-        <v>46284.58333333334</v>
+        <v>46294.58333333334</v>
       </c>
       <c r="B154">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="2">
-        <v>46284.59375</v>
+        <v>46294.59375</v>
       </c>
       <c r="B155">
-        <v>240</v>
+        <v>251</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="2">
-        <v>46284.60416666666</v>
+        <v>46294.60416666666</v>
       </c>
       <c r="B156">
-        <v>241</v>
+        <v>233</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="2">
-        <v>46284.61458333334</v>
+        <v>46294.61458333334</v>
       </c>
       <c r="B157">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="2">
-        <v>46284.625</v>
+        <v>46294.625</v>
       </c>
       <c r="B158">
-        <v>241</v>
+        <v>215</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="2">
-        <v>46284.63541666666</v>
+        <v>46294.63541666666</v>
       </c>
       <c r="B159">
-        <v>241</v>
+        <v>201</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="2">
-        <v>46284.64583333334</v>
+        <v>46294.64583333334</v>
       </c>
       <c r="B160">
-        <v>241</v>
+        <v>200</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="2">
-        <v>46284.65625</v>
+        <v>46294.65625</v>
       </c>
       <c r="B161">
-        <v>247</v>
+        <v>201</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="2">
-        <v>46284.66666666666</v>
+        <v>46294.66666666666</v>
       </c>
       <c r="B162">
-        <v>297</v>
+        <v>224</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="2">
-        <v>46284.67708333334</v>
+        <v>46294.67708333334</v>
       </c>
       <c r="B163">
-        <v>298</v>
+        <v>222</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="2">
-        <v>46284.6875</v>
+        <v>46294.6875</v>
       </c>
       <c r="B164">
-        <v>298</v>
+        <v>224</v>
       </c>
     </row>
     <row r="165" spans="1:2">
       <c r="A165" s="2">
-        <v>46284.69791666666</v>
+        <v>46294.69791666666</v>
       </c>
       <c r="B165">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="166" spans="1:2">
       <c r="A166" s="2">
-        <v>46284.70833333334</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="B166">
-        <v>443</v>
+        <v>534</v>
       </c>
     </row>
     <row r="167" spans="1:2">
       <c r="A167" s="2">
-        <v>46284.71875</v>
+        <v>46294.71875</v>
       </c>
       <c r="B167">
-        <v>457</v>
+        <v>566</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="2">
-        <v>46284.72916666666</v>
+        <v>46294.72916666666</v>
       </c>
       <c r="B168">
-        <v>459</v>
+        <v>576</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="2">
-        <v>46284.73958333334</v>
+        <v>46294.73958333334</v>
       </c>
       <c r="B169">
-        <v>464</v>
+        <v>749</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="2">
-        <v>46284.75</v>
+        <v>46294.75</v>
       </c>
       <c r="B170">
-        <v>678</v>
+        <v>890</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="2">
-        <v>46284.76041666666</v>
+        <v>46294.76041666666</v>
       </c>
       <c r="B171">
-        <v>696</v>
+        <v>856</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="2">
-        <v>46284.77083333334</v>
+        <v>46294.77083333334</v>
       </c>
       <c r="B172">
-        <v>694</v>
+        <v>856</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="2">
-        <v>46284.78125</v>
+        <v>46294.78125</v>
       </c>
       <c r="B173">
-        <v>695</v>
+        <v>853</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="2">
-        <v>46284.79166666666</v>
+        <v>46294.79166666666</v>
       </c>
       <c r="B174">
-        <v>636</v>
+        <v>747</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="2">
-        <v>46284.80208333334</v>
+        <v>46294.80208333334</v>
       </c>
       <c r="B175">
-        <v>632</v>
+        <v>746</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="2">
-        <v>46284.8125</v>
+        <v>46294.8125</v>
       </c>
       <c r="B176">
-        <v>633</v>
+        <v>746</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="2">
-        <v>46284.82291666666</v>
+        <v>46294.82291666666</v>
       </c>
       <c r="B177">
-        <v>631</v>
+        <v>745</v>
       </c>
     </row>
     <row r="178" spans="1:2">
       <c r="A178" s="2">
-        <v>46284.83333333334</v>
+        <v>46294.83333333334</v>
       </c>
       <c r="B178">
-        <v>631</v>
+        <v>675</v>
       </c>
     </row>
     <row r="179" spans="1:2">
       <c r="A179" s="2">
-        <v>46284.84375</v>
+        <v>46294.84375</v>
       </c>
       <c r="B179">
-        <v>630</v>
+        <v>678</v>
       </c>
     </row>
     <row r="180" spans="1:2">
       <c r="A180" s="2">
-        <v>46284.85416666666</v>
+        <v>46294.85416666666</v>
       </c>
       <c r="B180">
-        <v>631</v>
+        <v>636</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="2">
-        <v>46284.86458333334</v>
+        <v>46294.86458333334</v>
       </c>
       <c r="B181">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="2">
-        <v>46284.875</v>
+        <v>46294.875</v>
       </c>
       <c r="B182">
-        <v>566</v>
+        <v>498</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="2">
-        <v>46284.88541666666</v>
+        <v>46294.88541666666</v>
       </c>
       <c r="B183">
-        <v>561</v>
+        <v>487</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="2">
-        <v>46284.89583333334</v>
+        <v>46294.89583333334</v>
       </c>
       <c r="B184">
-        <v>564</v>
+        <v>487</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="2">
-        <v>46284.90625</v>
+        <v>46294.90625</v>
       </c>
       <c r="B185">
-        <v>560</v>
+        <v>483</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="2">
-        <v>46284.91666666666</v>
+        <v>46294.91666666666</v>
       </c>
       <c r="B186">
-        <v>580</v>
+        <v>327</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="2">
-        <v>46284.92708333334</v>
+        <v>46294.92708333334</v>
       </c>
       <c r="B187">
-        <v>577</v>
+        <v>303</v>
       </c>
     </row>
     <row r="188" spans="1:2">
       <c r="A188" s="2">
-        <v>46284.9375</v>
+        <v>46294.9375</v>
       </c>
       <c r="B188">
-        <v>579</v>
+        <v>313</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="2">
-        <v>46284.94791666666</v>
+        <v>46294.94791666666</v>
       </c>
       <c r="B189">
-        <v>575</v>
+        <v>312</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="2">
-        <v>46284.95833333334</v>
+        <v>46294.95833333334</v>
       </c>
       <c r="B190">
-        <v>563</v>
+        <v>285</v>
       </c>
     </row>
     <row r="191" spans="1:2">
       <c r="A191" s="2">
-        <v>46284.96875</v>
+        <v>46294.96875</v>
       </c>
       <c r="B191">
-        <v>560</v>
+        <v>281</v>
       </c>
     </row>
     <row r="192" spans="1:2">
       <c r="A192" s="2">
-        <v>46284.97916666666</v>
+        <v>46294.97916666666</v>
       </c>
       <c r="B192">
-        <v>562</v>
+        <v>282</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="2">
-        <v>46284.98958333334</v>
+        <v>46294.98958333334</v>
       </c>
       <c r="B193">
-        <v>564</v>
+        <v>277</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="2">
-        <v>46285</v>
+        <v>46295</v>
       </c>
       <c r="B194">
-        <v>616</v>
+        <v>229</v>
       </c>
     </row>
     <row r="195" spans="1:2">
       <c r="A195" s="2">
-        <v>46285.01041666666</v>
+        <v>46295.01041666666</v>
       </c>
       <c r="B195">
-        <v>616</v>
+        <v>231</v>
       </c>
     </row>
     <row r="196" spans="1:2">
       <c r="A196" s="2">
-        <v>46285.02083333334</v>
+        <v>46295.02083333334</v>
       </c>
       <c r="B196">
-        <v>617</v>
+        <v>230</v>
       </c>
     </row>
     <row r="197" spans="1:2">
       <c r="A197" s="2">
-        <v>46285.03125</v>
+        <v>46295.03125</v>
       </c>
       <c r="B197">
-        <v>617</v>
+        <v>229</v>
       </c>
     </row>
     <row r="198" spans="1:2">
       <c r="A198" s="2">
-        <v>46285.04166666666</v>
+        <v>46295.04166666666</v>
       </c>
       <c r="B198">
-        <v>518</v>
+        <v>227</v>
       </c>
     </row>
     <row r="199" spans="1:2">
       <c r="A199" s="2">
-        <v>46285.05208333334</v>
+        <v>46295.05208333334</v>
       </c>
       <c r="B199">
-        <v>503</v>
+        <v>227</v>
       </c>
     </row>
     <row r="200" spans="1:2">
       <c r="A200" s="2">
-        <v>46285.0625</v>
+        <v>46295.0625</v>
       </c>
       <c r="B200">
-        <v>502</v>
+        <v>227</v>
       </c>
     </row>
     <row r="201" spans="1:2">
       <c r="A201" s="2">
-        <v>46285.07291666666</v>
+        <v>46295.07291666666</v>
       </c>
       <c r="B201">
-        <v>502</v>
+        <v>227</v>
       </c>
     </row>
     <row r="202" spans="1:2">
       <c r="A202" s="2">
-        <v>46285.08333333334</v>
+        <v>46295.08333333334</v>
       </c>
       <c r="B202">
-        <v>502</v>
+        <v>220</v>
       </c>
     </row>
     <row r="203" spans="1:2">
       <c r="A203" s="2">
-        <v>46285.09375</v>
+        <v>46295.09375</v>
       </c>
       <c r="B203">
-        <v>502</v>
+        <v>219</v>
       </c>
     </row>
     <row r="204" spans="1:2">
       <c r="A204" s="2">
-        <v>46285.10416666666</v>
+        <v>46295.10416666666</v>
       </c>
       <c r="B204">
-        <v>502</v>
+        <v>219</v>
       </c>
     </row>
     <row r="205" spans="1:2">
       <c r="A205" s="2">
-        <v>46285.11458333334</v>
+        <v>46295.11458333334</v>
       </c>
       <c r="B205">
-        <v>502</v>
+        <v>219</v>
       </c>
     </row>
     <row r="206" spans="1:2">
       <c r="A206" s="2">
-        <v>46285.125</v>
+        <v>46295.125</v>
       </c>
       <c r="B206">
-        <v>502</v>
+        <v>224</v>
       </c>
     </row>
     <row r="207" spans="1:2">
       <c r="A207" s="2">
-        <v>46285.13541666666</v>
+        <v>46295.13541666666</v>
       </c>
       <c r="B207">
-        <v>501</v>
+        <v>224</v>
       </c>
     </row>
     <row r="208" spans="1:2">
       <c r="A208" s="2">
-        <v>46285.14583333334</v>
+        <v>46295.14583333334</v>
       </c>
       <c r="B208">
-        <v>502</v>
+        <v>224</v>
       </c>
     </row>
     <row r="209" spans="1:2">
       <c r="A209" s="2">
-        <v>46285.15625</v>
+        <v>46295.15625</v>
       </c>
       <c r="B209">
-        <v>501</v>
+        <v>224</v>
       </c>
     </row>
     <row r="210" spans="1:2">
       <c r="A210" s="2">
-        <v>46285.16666666666</v>
+        <v>46295.16666666666</v>
       </c>
       <c r="B210">
-        <v>510</v>
+        <v>225</v>
       </c>
     </row>
     <row r="211" spans="1:2">
       <c r="A211" s="2">
-        <v>46285.17708333334</v>
+        <v>46295.17708333334</v>
       </c>
       <c r="B211">
-        <v>515</v>
+        <v>244</v>
       </c>
     </row>
     <row r="212" spans="1:2">
       <c r="A212" s="2">
-        <v>46285.1875</v>
+        <v>46295.1875</v>
       </c>
       <c r="B212">
-        <v>515</v>
+        <v>245</v>
       </c>
     </row>
     <row r="213" spans="1:2">
       <c r="A213" s="2">
-        <v>46285.19791666666</v>
+        <v>46295.19791666666</v>
       </c>
       <c r="B213">
-        <v>515</v>
+        <v>246</v>
       </c>
     </row>
     <row r="214" spans="1:2">
       <c r="A214" s="2">
-        <v>46285.20833333334</v>
+        <v>46295.20833333334</v>
       </c>
       <c r="B214">
-        <v>475</v>
+        <v>297</v>
       </c>
     </row>
     <row r="215" spans="1:2">
       <c r="A215" s="2">
-        <v>46285.21875</v>
+        <v>46295.21875</v>
       </c>
       <c r="B215">
-        <v>471</v>
+        <v>297</v>
       </c>
     </row>
     <row r="216" spans="1:2">
       <c r="A216" s="2">
-        <v>46285.22916666666</v>
+        <v>46295.22916666666</v>
       </c>
       <c r="B216">
-        <v>471</v>
+        <v>298</v>
       </c>
     </row>
     <row r="217" spans="1:2">
       <c r="A217" s="2">
-        <v>46285.23958333334</v>
+        <v>46295.23958333334</v>
       </c>
       <c r="B217">
-        <v>471</v>
+        <v>302</v>
       </c>
     </row>
     <row r="218" spans="1:2">
       <c r="A218" s="2">
-        <v>46285.25</v>
+        <v>46295.25</v>
       </c>
       <c r="B218">
-        <v>512</v>
+        <v>600</v>
       </c>
     </row>
     <row r="219" spans="1:2">
       <c r="A219" s="2">
-        <v>46285.26041666666</v>
+        <v>46295.26041666666</v>
       </c>
       <c r="B219">
-        <v>513</v>
+        <v>649</v>
       </c>
     </row>
     <row r="220" spans="1:2">
       <c r="A220" s="2">
-        <v>46285.27083333334</v>
+        <v>46295.27083333334</v>
       </c>
       <c r="B220">
-        <v>513</v>
+        <v>643</v>
       </c>
     </row>
     <row r="221" spans="1:2">
       <c r="A221" s="2">
-        <v>46285.28125</v>
+        <v>46295.28125</v>
       </c>
       <c r="B221">
-        <v>511</v>
+        <v>645</v>
       </c>
     </row>
     <row r="222" spans="1:2">
       <c r="A222" s="2">
-        <v>46285.29166666666</v>
+        <v>46295.29166666666</v>
       </c>
       <c r="B222">
-        <v>276</v>
+        <v>623</v>
       </c>
     </row>
     <row r="223" spans="1:2">
       <c r="A223" s="2">
-        <v>46285.30208333334</v>
+        <v>46295.30208333334</v>
       </c>
       <c r="B223">
-        <v>254</v>
+        <v>636</v>
       </c>
     </row>
     <row r="224" spans="1:2">
       <c r="A224" s="2">
-        <v>46285.3125</v>
+        <v>46295.3125</v>
       </c>
       <c r="B224">
-        <v>254</v>
+        <v>638</v>
       </c>
     </row>
     <row r="225" spans="1:2">
       <c r="A225" s="2">
-        <v>46285.32291666666</v>
+        <v>46295.32291666666</v>
       </c>
       <c r="B225">
-        <v>254</v>
+        <v>637</v>
       </c>
     </row>
     <row r="226" spans="1:2">
       <c r="A226" s="2">
-        <v>46285.33333333334</v>
+        <v>46295.33333333334</v>
       </c>
       <c r="B226">
-        <v>246</v>
+        <v>461</v>
       </c>
     </row>
     <row r="227" spans="1:2">
       <c r="A227" s="2">
-        <v>46285.34375</v>
+        <v>46295.34375</v>
       </c>
       <c r="B227">
-        <v>244</v>
+        <v>418</v>
       </c>
     </row>
     <row r="228" spans="1:2">
       <c r="A228" s="2">
-        <v>46285.35416666666</v>
+        <v>46295.35416666666</v>
       </c>
       <c r="B228">
-        <v>244</v>
+        <v>420</v>
       </c>
     </row>
     <row r="229" spans="1:2">
       <c r="A229" s="2">
-        <v>46285.36458333334</v>
+        <v>46295.36458333334</v>
       </c>
       <c r="B229">
-        <v>245</v>
+        <v>417</v>
       </c>
     </row>
     <row r="230" spans="1:2">
       <c r="A230" s="2">
-        <v>46285.375</v>
+        <v>46295.375</v>
       </c>
       <c r="B230">
-        <v>241</v>
+        <v>319</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46295.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46295.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for GCSP
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B327"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,375 +394,375 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B2">
-        <v>227</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46303.01041666666</v>
+        <v>46304.01041666666</v>
       </c>
       <c r="B3">
-        <v>214</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46303.02083333334</v>
+        <v>46304.02083333334</v>
       </c>
       <c r="B4">
-        <v>215</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46303.03125</v>
+        <v>46304.03125</v>
       </c>
       <c r="B5">
-        <v>215</v>
+        <v>377</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46303.04166666666</v>
+        <v>46304.04166666666</v>
       </c>
       <c r="B6">
-        <v>284</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46303.05208333334</v>
+        <v>46304.05208333334</v>
       </c>
       <c r="B7">
-        <v>286</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46303.0625</v>
+        <v>46304.0625</v>
       </c>
       <c r="B8">
-        <v>286</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46303.07291666666</v>
+        <v>46304.07291666666</v>
       </c>
       <c r="B9">
-        <v>285</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46303.08333333334</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="B10">
-        <v>286</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46303.09375</v>
+        <v>46304.09375</v>
       </c>
       <c r="B11">
-        <v>286</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46303.10416666666</v>
+        <v>46304.10416666666</v>
       </c>
       <c r="B12">
-        <v>285</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46303.11458333334</v>
+        <v>46304.11458333334</v>
       </c>
       <c r="B13">
-        <v>284</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46303.125</v>
+        <v>46304.125</v>
       </c>
       <c r="B14">
-        <v>285</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46303.13541666666</v>
+        <v>46304.13541666666</v>
       </c>
       <c r="B15">
-        <v>284</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46303.14583333334</v>
+        <v>46304.14583333334</v>
       </c>
       <c r="B16">
-        <v>284</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46303.15625</v>
+        <v>46304.15625</v>
       </c>
       <c r="B17">
-        <v>284</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46303.16666666666</v>
+        <v>46304.16666666666</v>
       </c>
       <c r="B18">
-        <v>281</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46303.17708333334</v>
+        <v>46304.17708333334</v>
       </c>
       <c r="B19">
-        <v>280</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46303.1875</v>
+        <v>46304.1875</v>
       </c>
       <c r="B20">
-        <v>295</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46303.19791666666</v>
+        <v>46304.19791666666</v>
       </c>
       <c r="B21">
-        <v>299</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46303.20833333334</v>
+        <v>46304.20833333334</v>
       </c>
       <c r="B22">
-        <v>447</v>
+        <v>547</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46303.21875</v>
+        <v>46304.21875</v>
       </c>
       <c r="B23">
-        <v>456</v>
+        <v>558</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46303.22916666666</v>
+        <v>46304.22916666666</v>
       </c>
       <c r="B24">
-        <v>453</v>
+        <v>576</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46303.23958333334</v>
+        <v>46304.23958333334</v>
       </c>
       <c r="B25">
-        <v>457</v>
+        <v>582</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46303.25</v>
+        <v>46304.25</v>
       </c>
       <c r="B26">
-        <v>643</v>
+        <v>583</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46303.26041666666</v>
+        <v>46304.26041666666</v>
       </c>
       <c r="B27">
-        <v>656</v>
+        <v>566</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46303.27083333334</v>
+        <v>46304.27083333334</v>
       </c>
       <c r="B28">
-        <v>638</v>
+        <v>591</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46303.28125</v>
+        <v>46304.28125</v>
       </c>
       <c r="B29">
-        <v>644</v>
+        <v>544</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46303.29166666666</v>
+        <v>46304.29166666666</v>
       </c>
       <c r="B30">
-        <v>695</v>
+        <v>526</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46303.30208333334</v>
+        <v>46304.30208333334</v>
       </c>
       <c r="B31">
-        <v>681</v>
+        <v>514</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46303.3125</v>
+        <v>46304.3125</v>
       </c>
       <c r="B32">
-        <v>702</v>
+        <v>517</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46303.32291666666</v>
+        <v>46304.32291666666</v>
       </c>
       <c r="B33">
-        <v>702</v>
+        <v>519</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46303.33333333334</v>
+        <v>46304.33333333334</v>
       </c>
       <c r="B34">
-        <v>658</v>
+        <v>476</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46303.34375</v>
+        <v>46304.34375</v>
       </c>
       <c r="B35">
-        <v>681</v>
+        <v>472</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46303.35416666666</v>
+        <v>46304.35416666666</v>
       </c>
       <c r="B36">
-        <v>682</v>
+        <v>472</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46303.36458333334</v>
+        <v>46304.36458333334</v>
       </c>
       <c r="B37">
-        <v>678</v>
+        <v>472</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46303.375</v>
+        <v>46304.375</v>
       </c>
       <c r="B38">
-        <v>284</v>
+        <v>239</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46303.38541666666</v>
+        <v>46304.38541666666</v>
       </c>
       <c r="B39">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46303.39583333334</v>
+        <v>46304.39583333334</v>
       </c>
       <c r="B40">
-        <v>196</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46303.40625</v>
+        <v>46304.40625</v>
       </c>
       <c r="B41">
-        <v>194</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46303.41666666666</v>
+        <v>46304.41666666666</v>
       </c>
       <c r="B42">
-        <v>206</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46303.42708333334</v>
+        <v>46304.42708333334</v>
       </c>
       <c r="B43">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46303.4375</v>
+        <v>46304.4375</v>
       </c>
       <c r="B44">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46303.44791666666</v>
+        <v>46304.44791666666</v>
       </c>
       <c r="B45">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46303.45833333334</v>
+        <v>46304.45833333334</v>
       </c>
       <c r="B46">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46303.46875</v>
+        <v>46304.46875</v>
       </c>
       <c r="B47">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46303.47916666666</v>
+        <v>46304.47916666666</v>
       </c>
       <c r="B48">
         <v>204</v>
@@ -770,87 +770,87 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46303.48958333334</v>
+        <v>46304.48958333334</v>
       </c>
       <c r="B49">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46303.5</v>
+        <v>46304.5</v>
       </c>
       <c r="B50">
-        <v>217</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46303.51041666666</v>
+        <v>46304.51041666666</v>
       </c>
       <c r="B51">
-        <v>222</v>
+        <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46303.52083333334</v>
+        <v>46304.52083333334</v>
       </c>
       <c r="B52">
-        <v>223</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46303.53125</v>
+        <v>46304.53125</v>
       </c>
       <c r="B53">
-        <v>226</v>
+        <v>200</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46303.54166666666</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="B54">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46303.55208333334</v>
+        <v>46304.55208333334</v>
       </c>
       <c r="B55">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46303.5625</v>
+        <v>46304.5625</v>
       </c>
       <c r="B56">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46303.57291666666</v>
+        <v>46304.57291666666</v>
       </c>
       <c r="B57">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46303.58333333334</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="B58">
-        <v>216</v>
+        <v>198</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46303.59375</v>
+        <v>46304.59375</v>
       </c>
       <c r="B59">
         <v>215</v>
@@ -858,578 +858,2146 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46303.60416666666</v>
+        <v>46304.60416666666</v>
       </c>
       <c r="B60">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46303.61458333334</v>
+        <v>46304.61458333334</v>
       </c>
       <c r="B61">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46303.625</v>
+        <v>46304.625</v>
       </c>
       <c r="B62">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46303.63541666666</v>
+        <v>46304.63541666666</v>
       </c>
       <c r="B63">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46303.64583333334</v>
+        <v>46304.64583333334</v>
       </c>
       <c r="B64">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46303.65625</v>
+        <v>46304.65625</v>
       </c>
       <c r="B65">
-        <v>188</v>
+        <v>202</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46303.66666666666</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="B66">
-        <v>416</v>
+        <v>482</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46303.67708333334</v>
+        <v>46304.67708333334</v>
       </c>
       <c r="B67">
-        <v>421</v>
+        <v>498</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46303.6875</v>
+        <v>46304.6875</v>
       </c>
       <c r="B68">
-        <v>442</v>
+        <v>498</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46303.69791666666</v>
+        <v>46304.69791666666</v>
       </c>
       <c r="B69">
-        <v>463</v>
+        <v>509</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46303.70833333334</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="B70">
-        <v>463</v>
+        <v>561</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46303.71875</v>
+        <v>46304.71875</v>
       </c>
       <c r="B71">
-        <v>477</v>
+        <v>566</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46303.72916666666</v>
+        <v>46304.72916666666</v>
       </c>
       <c r="B72">
-        <v>532</v>
+        <v>555</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46303.73958333334</v>
+        <v>46304.73958333334</v>
       </c>
       <c r="B73">
-        <v>533</v>
+        <v>551</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46303.75</v>
+        <v>46304.75</v>
       </c>
       <c r="B74">
-        <v>529</v>
+        <v>665</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46303.76041666666</v>
+        <v>46304.76041666666</v>
       </c>
       <c r="B75">
-        <v>532</v>
+        <v>670</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46303.77083333334</v>
+        <v>46304.77083333334</v>
       </c>
       <c r="B76">
-        <v>527</v>
+        <v>671</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46303.78125</v>
+        <v>46304.78125</v>
       </c>
       <c r="B77">
-        <v>530</v>
+        <v>670</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46303.79166666666</v>
+        <v>46304.79166666666</v>
       </c>
       <c r="B78">
-        <v>633</v>
+        <v>660</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46303.80208333334</v>
+        <v>46304.80208333334</v>
       </c>
       <c r="B79">
-        <v>639</v>
+        <v>661</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46303.8125</v>
+        <v>46304.8125</v>
       </c>
       <c r="B80">
-        <v>627</v>
+        <v>659</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46303.82291666666</v>
+        <v>46304.82291666666</v>
       </c>
       <c r="B81">
-        <v>626</v>
+        <v>660</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46303.83333333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="B82">
-        <v>642</v>
+        <v>646</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46303.84375</v>
+        <v>46304.84375</v>
       </c>
       <c r="B83">
-        <v>649</v>
+        <v>645</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46303.85416666666</v>
+        <v>46304.85416666666</v>
       </c>
       <c r="B84">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46303.86458333334</v>
+        <v>46304.86458333334</v>
       </c>
       <c r="B85">
-        <v>651</v>
+        <v>649</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46303.875</v>
+        <v>46304.875</v>
       </c>
       <c r="B86">
-        <v>612</v>
+        <v>638</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46303.88541666666</v>
+        <v>46304.88541666666</v>
       </c>
       <c r="B87">
-        <v>611</v>
+        <v>636</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46303.89583333334</v>
+        <v>46304.89583333334</v>
       </c>
       <c r="B88">
-        <v>621</v>
+        <v>638</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46303.90625</v>
+        <v>46304.90625</v>
       </c>
       <c r="B89">
-        <v>621</v>
+        <v>634</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46303.91666666666</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="B90">
-        <v>540</v>
+        <v>609</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46303.92708333334</v>
+        <v>46304.92708333334</v>
       </c>
       <c r="B91">
-        <v>535</v>
+        <v>603</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46303.9375</v>
+        <v>46304.9375</v>
       </c>
       <c r="B92">
-        <v>534</v>
+        <v>604</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46303.94791666666</v>
+        <v>46304.94791666666</v>
       </c>
       <c r="B93">
-        <v>533</v>
+        <v>604</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46303.95833333334</v>
+        <v>46304.95833333334</v>
       </c>
       <c r="B94">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46303.96875</v>
+        <v>46304.96875</v>
       </c>
       <c r="B95">
-        <v>399</v>
+        <v>406</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46303.97916666666</v>
+        <v>46304.97916666666</v>
       </c>
       <c r="B96">
-        <v>402</v>
+        <v>453</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46303.98958333334</v>
+        <v>46304.98958333334</v>
       </c>
       <c r="B97">
-        <v>402</v>
+        <v>467</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B98">
-        <v>381</v>
+        <v>449</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46304.01041666666</v>
+        <v>46305.01041666666</v>
       </c>
       <c r="B99">
-        <v>380</v>
+        <v>422</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46304.02083333334</v>
+        <v>46305.02083333334</v>
       </c>
       <c r="B100">
-        <v>378</v>
+        <v>414</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46304.03125</v>
+        <v>46305.03125</v>
       </c>
       <c r="B101">
-        <v>377</v>
+        <v>397</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46304.04166666666</v>
+        <v>46305.04166666666</v>
       </c>
       <c r="B102">
-        <v>309</v>
+        <v>399</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46304.05208333334</v>
+        <v>46305.05208333334</v>
       </c>
       <c r="B103">
-        <v>305</v>
+        <v>399</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46304.0625</v>
+        <v>46305.0625</v>
       </c>
       <c r="B104">
-        <v>305</v>
+        <v>399</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46304.07291666666</v>
+        <v>46305.07291666666</v>
       </c>
       <c r="B105">
-        <v>305</v>
+        <v>398</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46304.08333333334</v>
+        <v>46305.08333333334</v>
       </c>
       <c r="B106">
-        <v>181</v>
+        <v>395</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46304.09375</v>
+        <v>46305.09375</v>
       </c>
       <c r="B107">
-        <v>176</v>
+        <v>392</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46304.10416666666</v>
+        <v>46305.10416666666</v>
       </c>
       <c r="B108">
-        <v>176</v>
+        <v>393</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46304.11458333334</v>
+        <v>46305.11458333334</v>
       </c>
       <c r="B109">
-        <v>175</v>
+        <v>392</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46304.125</v>
+        <v>46305.125</v>
       </c>
       <c r="B110">
-        <v>173</v>
+        <v>391</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46304.13541666666</v>
+        <v>46305.13541666666</v>
       </c>
       <c r="B111">
-        <v>196</v>
+        <v>391</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46304.14583333334</v>
+        <v>46305.14583333334</v>
       </c>
       <c r="B112">
-        <v>201</v>
+        <v>392</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46304.15625</v>
+        <v>46305.15625</v>
       </c>
       <c r="B113">
-        <v>217</v>
+        <v>392</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46304.16666666666</v>
+        <v>46305.16666666666</v>
       </c>
       <c r="B114">
-        <v>310</v>
+        <v>419</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46304.17708333334</v>
+        <v>46305.17708333334</v>
       </c>
       <c r="B115">
-        <v>316</v>
+        <v>441</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46304.1875</v>
+        <v>46305.1875</v>
       </c>
       <c r="B116">
-        <v>317</v>
+        <v>442</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46304.19791666666</v>
+        <v>46305.19791666666</v>
       </c>
       <c r="B117">
-        <v>322</v>
+        <v>442</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46304.20833333334</v>
+        <v>46305.20833333334</v>
       </c>
       <c r="B118">
-        <v>547</v>
+        <v>486</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46304.21875</v>
+        <v>46305.21875</v>
       </c>
       <c r="B119">
-        <v>558</v>
+        <v>493</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46304.22916666666</v>
+        <v>46305.22916666666</v>
       </c>
       <c r="B120">
-        <v>576</v>
+        <v>442</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46304.23958333334</v>
+        <v>46305.23958333334</v>
       </c>
       <c r="B121">
-        <v>582</v>
+        <v>439</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46304.25</v>
+        <v>46305.25</v>
       </c>
       <c r="B122">
-        <v>583</v>
+        <v>509</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46304.26041666666</v>
+        <v>46305.26041666666</v>
       </c>
       <c r="B123">
-        <v>566</v>
+        <v>524</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46304.27083333334</v>
+        <v>46305.27083333334</v>
       </c>
       <c r="B124">
-        <v>591</v>
+        <v>518</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46304.28125</v>
+        <v>46305.28125</v>
       </c>
       <c r="B125">
-        <v>544</v>
+        <v>517</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46304.29166666666</v>
+        <v>46305.29166666666</v>
       </c>
       <c r="B126">
-        <v>526</v>
+        <v>477</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46304.30208333334</v>
+        <v>46305.30208333334</v>
       </c>
       <c r="B127">
-        <v>514</v>
+        <v>476</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46304.3125</v>
+        <v>46305.3125</v>
       </c>
       <c r="B128">
-        <v>517</v>
+        <v>477</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46304.32291666666</v>
+        <v>46305.32291666666</v>
       </c>
       <c r="B129">
-        <v>519</v>
+        <v>475</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46304.33333333334</v>
+        <v>46305.33333333334</v>
       </c>
       <c r="B130">
-        <v>476</v>
+        <v>461</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46304.34375</v>
+        <v>46305.34375</v>
       </c>
       <c r="B131">
-        <v>472</v>
+        <v>458</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="2">
+        <v>46305.35416666666</v>
+      </c>
+      <c r="B132">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="2">
+        <v>46305.36458333334</v>
+      </c>
+      <c r="B133">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="2">
+        <v>46305.375</v>
+      </c>
+      <c r="B134">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="2">
+        <v>46305.38541666666</v>
+      </c>
+      <c r="B135">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="2">
+        <v>46305.39583333334</v>
+      </c>
+      <c r="B136">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="2">
+        <v>46305.40625</v>
+      </c>
+      <c r="B137">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="2">
+        <v>46305.41666666666</v>
+      </c>
+      <c r="B138">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="2">
+        <v>46305.42708333334</v>
+      </c>
+      <c r="B139">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="2">
+        <v>46305.4375</v>
+      </c>
+      <c r="B140">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="2">
+        <v>46305.44791666666</v>
+      </c>
+      <c r="B141">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="2">
+        <v>46305.45833333334</v>
+      </c>
+      <c r="B142">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="2">
+        <v>46305.46875</v>
+      </c>
+      <c r="B143">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="2">
+        <v>46305.47916666666</v>
+      </c>
+      <c r="B144">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="2">
+        <v>46305.48958333334</v>
+      </c>
+      <c r="B145">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="2">
+        <v>46305.5</v>
+      </c>
+      <c r="B146">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="2">
+        <v>46305.51041666666</v>
+      </c>
+      <c r="B147">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="2">
+        <v>46305.52083333334</v>
+      </c>
+      <c r="B148">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="2">
+        <v>46305.53125</v>
+      </c>
+      <c r="B149">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="2">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="B150">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46305.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46305.5625</v>
+      </c>
+      <c r="B152">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46305.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46305.59375</v>
+      </c>
+      <c r="B155">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="2">
+        <v>46305.60416666666</v>
+      </c>
+      <c r="B156">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="2">
+        <v>46305.61458333334</v>
+      </c>
+      <c r="B157">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="2">
+        <v>46305.625</v>
+      </c>
+      <c r="B158">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="2">
+        <v>46305.63541666666</v>
+      </c>
+      <c r="B159">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="2">
+        <v>46305.64583333334</v>
+      </c>
+      <c r="B160">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="2">
+        <v>46305.65625</v>
+      </c>
+      <c r="B161">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="2">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="B162">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2">
+        <v>46305.67708333334</v>
+      </c>
+      <c r="B163">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="2">
+        <v>46305.6875</v>
+      </c>
+      <c r="B164">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2">
+        <v>46305.69791666666</v>
+      </c>
+      <c r="B165">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="B166">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="2">
+        <v>46305.71875</v>
+      </c>
+      <c r="B167">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="2">
+        <v>46305.72916666666</v>
+      </c>
+      <c r="B168">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="2">
+        <v>46305.73958333334</v>
+      </c>
+      <c r="B169">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="2">
+        <v>46305.75</v>
+      </c>
+      <c r="B170">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="2">
+        <v>46305.76041666666</v>
+      </c>
+      <c r="B171">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="2">
+        <v>46305.77083333334</v>
+      </c>
+      <c r="B172">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="2">
+        <v>46305.78125</v>
+      </c>
+      <c r="B173">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="2">
+        <v>46305.79166666666</v>
+      </c>
+      <c r="B174">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="2">
+        <v>46305.80208333334</v>
+      </c>
+      <c r="B175">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="2">
+        <v>46305.8125</v>
+      </c>
+      <c r="B176">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="2">
+        <v>46305.82291666666</v>
+      </c>
+      <c r="B177">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="2">
+        <v>46305.83333333334</v>
+      </c>
+      <c r="B178">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="2">
+        <v>46305.84375</v>
+      </c>
+      <c r="B179">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="2">
+        <v>46305.85416666666</v>
+      </c>
+      <c r="B180">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="2">
+        <v>46305.86458333334</v>
+      </c>
+      <c r="B181">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="2">
+        <v>46305.875</v>
+      </c>
+      <c r="B182">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="2">
+        <v>46305.88541666666</v>
+      </c>
+      <c r="B183">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="2">
+        <v>46305.89583333334</v>
+      </c>
+      <c r="B184">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="2">
+        <v>46305.90625</v>
+      </c>
+      <c r="B185">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="2">
+        <v>46305.91666666666</v>
+      </c>
+      <c r="B186">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="2">
+        <v>46305.92708333334</v>
+      </c>
+      <c r="B187">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2">
+        <v>46305.9375</v>
+      </c>
+      <c r="B188">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="2">
+        <v>46305.94791666666</v>
+      </c>
+      <c r="B189">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2">
+        <v>46305.95833333334</v>
+      </c>
+      <c r="B190">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2">
+        <v>46305.96875</v>
+      </c>
+      <c r="B191">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="2">
+        <v>46305.97916666666</v>
+      </c>
+      <c r="B192">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2">
+        <v>46305.98958333334</v>
+      </c>
+      <c r="B193">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="2">
+        <v>46306</v>
+      </c>
+      <c r="B194">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="2">
+        <v>46306.01041666666</v>
+      </c>
+      <c r="B195">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="2">
+        <v>46306.02083333334</v>
+      </c>
+      <c r="B196">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="2">
+        <v>46306.03125</v>
+      </c>
+      <c r="B197">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="2">
+        <v>46306.04166666666</v>
+      </c>
+      <c r="B198">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="2">
+        <v>46306.05208333334</v>
+      </c>
+      <c r="B199">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="2">
+        <v>46306.0625</v>
+      </c>
+      <c r="B200">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" s="2">
+        <v>46306.07291666666</v>
+      </c>
+      <c r="B201">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="2">
+        <v>46306.08333333334</v>
+      </c>
+      <c r="B202">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" s="2">
+        <v>46306.09375</v>
+      </c>
+      <c r="B203">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" s="2">
+        <v>46306.10416666666</v>
+      </c>
+      <c r="B204">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" s="2">
+        <v>46306.11458333334</v>
+      </c>
+      <c r="B205">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" s="2">
+        <v>46306.125</v>
+      </c>
+      <c r="B206">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" s="2">
+        <v>46306.13541666666</v>
+      </c>
+      <c r="B207">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" s="2">
+        <v>46306.14583333334</v>
+      </c>
+      <c r="B208">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" s="2">
+        <v>46306.15625</v>
+      </c>
+      <c r="B209">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" s="2">
+        <v>46306.16666666666</v>
+      </c>
+      <c r="B210">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" s="2">
+        <v>46306.17708333334</v>
+      </c>
+      <c r="B211">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" s="2">
+        <v>46306.1875</v>
+      </c>
+      <c r="B212">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" s="2">
+        <v>46306.19791666666</v>
+      </c>
+      <c r="B213">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" s="2">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="B214">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" s="2">
+        <v>46306.21875</v>
+      </c>
+      <c r="B215">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" s="2">
+        <v>46306.22916666666</v>
+      </c>
+      <c r="B216">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" s="2">
+        <v>46306.23958333334</v>
+      </c>
+      <c r="B217">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" s="2">
+        <v>46306.25</v>
+      </c>
+      <c r="B218">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" s="2">
+        <v>46306.26041666666</v>
+      </c>
+      <c r="B219">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" s="2">
+        <v>46306.27083333334</v>
+      </c>
+      <c r="B220">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" s="2">
+        <v>46306.28125</v>
+      </c>
+      <c r="B221">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" s="2">
+        <v>46306.29166666666</v>
+      </c>
+      <c r="B222">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" s="2">
+        <v>46306.30208333334</v>
+      </c>
+      <c r="B223">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" s="2">
+        <v>46306.3125</v>
+      </c>
+      <c r="B224">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" s="2">
+        <v>46306.32291666666</v>
+      </c>
+      <c r="B225">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" s="2">
+        <v>46306.33333333334</v>
+      </c>
+      <c r="B226">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2">
+      <c r="A227" s="2">
+        <v>46306.34375</v>
+      </c>
+      <c r="B227">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2">
+      <c r="A228" s="2">
+        <v>46306.35416666666</v>
+      </c>
+      <c r="B228">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2">
+      <c r="A229" s="2">
+        <v>46306.36458333334</v>
+      </c>
+      <c r="B229">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2">
+      <c r="A230" s="2">
+        <v>46306.375</v>
+      </c>
+      <c r="B230">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" s="2">
+        <v>46306.38541666666</v>
+      </c>
+      <c r="B231">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2">
+      <c r="A232" s="2">
+        <v>46306.39583333334</v>
+      </c>
+      <c r="B232">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2">
+      <c r="A233" s="2">
+        <v>46306.40625</v>
+      </c>
+      <c r="B233">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2">
+      <c r="A234" s="2">
+        <v>46306.41666666666</v>
+      </c>
+      <c r="B234">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2">
+      <c r="A235" s="2">
+        <v>46306.42708333334</v>
+      </c>
+      <c r="B235">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2">
+      <c r="A236" s="2">
+        <v>46306.4375</v>
+      </c>
+      <c r="B236">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2">
+      <c r="A237" s="2">
+        <v>46306.44791666666</v>
+      </c>
+      <c r="B237">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2">
+      <c r="A238" s="2">
+        <v>46306.45833333334</v>
+      </c>
+      <c r="B238">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2">
+      <c r="A239" s="2">
+        <v>46306.46875</v>
+      </c>
+      <c r="B239">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2">
+      <c r="A240" s="2">
+        <v>46306.47916666666</v>
+      </c>
+      <c r="B240">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2">
+      <c r="A241" s="2">
+        <v>46306.48958333334</v>
+      </c>
+      <c r="B241">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2">
+      <c r="A242" s="2">
+        <v>46306.5</v>
+      </c>
+      <c r="B242">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2">
+      <c r="A243" s="2">
+        <v>46306.51041666666</v>
+      </c>
+      <c r="B243">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2">
+      <c r="A244" s="2">
+        <v>46306.52083333334</v>
+      </c>
+      <c r="B244">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2">
+      <c r="A245" s="2">
+        <v>46306.53125</v>
+      </c>
+      <c r="B245">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2">
+      <c r="A246" s="2">
+        <v>46306.54166666666</v>
+      </c>
+      <c r="B246">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2">
+      <c r="A247" s="2">
+        <v>46306.55208333334</v>
+      </c>
+      <c r="B247">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2">
+      <c r="A248" s="2">
+        <v>46306.5625</v>
+      </c>
+      <c r="B248">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2">
+      <c r="A249" s="2">
+        <v>46306.57291666666</v>
+      </c>
+      <c r="B249">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2">
+      <c r="A250" s="2">
+        <v>46306.58333333334</v>
+      </c>
+      <c r="B250">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2">
+      <c r="A251" s="2">
+        <v>46306.59375</v>
+      </c>
+      <c r="B251">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2">
+      <c r="A252" s="2">
+        <v>46306.60416666666</v>
+      </c>
+      <c r="B252">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2">
+      <c r="A253" s="2">
+        <v>46306.61458333334</v>
+      </c>
+      <c r="B253">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2">
+      <c r="A254" s="2">
+        <v>46306.625</v>
+      </c>
+      <c r="B254">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2">
+      <c r="A255" s="2">
+        <v>46306.63541666666</v>
+      </c>
+      <c r="B255">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2">
+      <c r="A256" s="2">
+        <v>46306.64583333334</v>
+      </c>
+      <c r="B256">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2">
+      <c r="A257" s="2">
+        <v>46306.65625</v>
+      </c>
+      <c r="B257">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2">
+      <c r="A258" s="2">
+        <v>46306.66666666666</v>
+      </c>
+      <c r="B258">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2">
+      <c r="A259" s="2">
+        <v>46306.67708333334</v>
+      </c>
+      <c r="B259">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2">
+      <c r="A260" s="2">
+        <v>46306.6875</v>
+      </c>
+      <c r="B260">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2">
+      <c r="A261" s="2">
+        <v>46306.69791666666</v>
+      </c>
+      <c r="B261">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2">
+      <c r="A262" s="2">
+        <v>46306.70833333334</v>
+      </c>
+      <c r="B262">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2">
+      <c r="A263" s="2">
+        <v>46306.71875</v>
+      </c>
+      <c r="B263">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2">
+      <c r="A264" s="2">
+        <v>46306.72916666666</v>
+      </c>
+      <c r="B264">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2">
+      <c r="A265" s="2">
+        <v>46306.73958333334</v>
+      </c>
+      <c r="B265">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2">
+      <c r="A266" s="2">
+        <v>46306.75</v>
+      </c>
+      <c r="B266">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2">
+      <c r="A267" s="2">
+        <v>46306.76041666666</v>
+      </c>
+      <c r="B267">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2">
+      <c r="A268" s="2">
+        <v>46306.77083333334</v>
+      </c>
+      <c r="B268">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2">
+      <c r="A269" s="2">
+        <v>46306.78125</v>
+      </c>
+      <c r="B269">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2">
+      <c r="A270" s="2">
+        <v>46306.79166666666</v>
+      </c>
+      <c r="B270">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2">
+      <c r="A271" s="2">
+        <v>46306.80208333334</v>
+      </c>
+      <c r="B271">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2">
+      <c r="A272" s="2">
+        <v>46306.8125</v>
+      </c>
+      <c r="B272">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2">
+      <c r="A273" s="2">
+        <v>46306.82291666666</v>
+      </c>
+      <c r="B273">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2">
+      <c r="A274" s="2">
+        <v>46306.83333333334</v>
+      </c>
+      <c r="B274">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2">
+      <c r="A275" s="2">
+        <v>46306.84375</v>
+      </c>
+      <c r="B275">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2">
+      <c r="A276" s="2">
+        <v>46306.85416666666</v>
+      </c>
+      <c r="B276">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2">
+      <c r="A277" s="2">
+        <v>46306.86458333334</v>
+      </c>
+      <c r="B277">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2">
+      <c r="A278" s="2">
+        <v>46306.875</v>
+      </c>
+      <c r="B278">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2">
+        <v>46306.88541666666</v>
+      </c>
+      <c r="B279">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="2">
+        <v>46306.89583333334</v>
+      </c>
+      <c r="B280">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="2">
+        <v>46306.90625</v>
+      </c>
+      <c r="B281">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="2">
+        <v>46306.91666666666</v>
+      </c>
+      <c r="B282">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="2">
+        <v>46306.92708333334</v>
+      </c>
+      <c r="B283">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="2">
+        <v>46306.9375</v>
+      </c>
+      <c r="B284">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="2">
+        <v>46306.94791666666</v>
+      </c>
+      <c r="B285">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="2">
+        <v>46306.95833333334</v>
+      </c>
+      <c r="B286">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="2">
+        <v>46306.96875</v>
+      </c>
+      <c r="B287">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="2">
+        <v>46306.97916666666</v>
+      </c>
+      <c r="B288">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="2">
+        <v>46306.98958333334</v>
+      </c>
+      <c r="B289">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="2">
+        <v>46307</v>
+      </c>
+      <c r="B290">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="2">
+        <v>46307.01041666666</v>
+      </c>
+      <c r="B291">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="2">
+        <v>46307.02083333334</v>
+      </c>
+      <c r="B292">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="2">
+        <v>46307.03125</v>
+      </c>
+      <c r="B293">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="2">
+        <v>46307.04166666666</v>
+      </c>
+      <c r="B294">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2">
+      <c r="A295" s="2">
+        <v>46307.05208333334</v>
+      </c>
+      <c r="B295">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2">
+      <c r="A296" s="2">
+        <v>46307.0625</v>
+      </c>
+      <c r="B296">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2">
+      <c r="A297" s="2">
+        <v>46307.07291666666</v>
+      </c>
+      <c r="B297">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2">
+      <c r="A298" s="2">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="B298">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2">
+      <c r="A299" s="2">
+        <v>46307.09375</v>
+      </c>
+      <c r="B299">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2">
+      <c r="A300" s="2">
+        <v>46307.10416666666</v>
+      </c>
+      <c r="B300">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2">
+      <c r="A301" s="2">
+        <v>46307.11458333334</v>
+      </c>
+      <c r="B301">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2">
+      <c r="A302" s="2">
+        <v>46307.125</v>
+      </c>
+      <c r="B302">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2">
+      <c r="A303" s="2">
+        <v>46307.13541666666</v>
+      </c>
+      <c r="B303">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2">
+      <c r="A304" s="2">
+        <v>46307.14583333334</v>
+      </c>
+      <c r="B304">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2">
+      <c r="A305" s="2">
+        <v>46307.15625</v>
+      </c>
+      <c r="B305">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2">
+      <c r="A306" s="2">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="B306">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2">
+      <c r="A307" s="2">
+        <v>46307.17708333334</v>
+      </c>
+      <c r="B307">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2">
+        <v>46307.1875</v>
+      </c>
+      <c r="B308">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2">
+        <v>46307.19791666666</v>
+      </c>
+      <c r="B309">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="B310">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2">
+        <v>46307.21875</v>
+      </c>
+      <c r="B311">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2">
+        <v>46307.22916666666</v>
+      </c>
+      <c r="B312">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2">
+        <v>46307.23958333334</v>
+      </c>
+      <c r="B313">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2">
+        <v>46307.25</v>
+      </c>
+      <c r="B314">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2">
+        <v>46307.26041666666</v>
+      </c>
+      <c r="B315">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2">
+        <v>46307.27083333334</v>
+      </c>
+      <c r="B316">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>46307.28125</v>
+      </c>
+      <c r="B317">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>46307.29166666666</v>
+      </c>
+      <c r="B318">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="2">
+        <v>46307.30208333334</v>
+      </c>
+      <c r="B319">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2">
+      <c r="A320" s="2">
+        <v>46307.3125</v>
+      </c>
+      <c r="B320">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2">
+      <c r="A321" s="2">
+        <v>46307.32291666666</v>
+      </c>
+      <c r="B321">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2">
+      <c r="A322" s="2">
+        <v>46307.33333333334</v>
+      </c>
+      <c r="B322">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2">
+      <c r="A323" s="2">
+        <v>46307.34375</v>
+      </c>
+      <c r="B323">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2">
+      <c r="A324" s="2">
+        <v>46307.35416666666</v>
+      </c>
+      <c r="B324">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2">
+      <c r="A325" s="2">
+        <v>46307.36458333334</v>
+      </c>
+      <c r="B325">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2">
+      <c r="A326" s="2">
+        <v>46307.375</v>
+      </c>
+      <c r="B326">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2">
+      <c r="A327" s="2">
+        <v>46307.38541666666</v>
+      </c>
+      <c r="B327">
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for Anto
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B150"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,1071 +394,1071 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B2">
-        <v>304</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46307.01041666666</v>
+        <v>46308.01041666666</v>
       </c>
       <c r="B3">
-        <v>307</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46307.02083333334</v>
+        <v>46308.02083333334</v>
       </c>
       <c r="B4">
-        <v>341</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46307.03125</v>
+        <v>46308.03125</v>
       </c>
       <c r="B5">
-        <v>341</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46307.04166666666</v>
+        <v>46308.04166666666</v>
       </c>
       <c r="B6">
-        <v>339</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46307.05208333334</v>
+        <v>46308.05208333334</v>
       </c>
       <c r="B7">
-        <v>309</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46307.0625</v>
+        <v>46308.0625</v>
       </c>
       <c r="B8">
-        <v>340</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46307.07291666666</v>
+        <v>46308.07291666666</v>
       </c>
       <c r="B9">
-        <v>323</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46307.08333333334</v>
+        <v>46308.08333333334</v>
       </c>
       <c r="B10">
-        <v>337</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46307.09375</v>
+        <v>46308.09375</v>
       </c>
       <c r="B11">
-        <v>327</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46307.10416666666</v>
+        <v>46308.10416666666</v>
       </c>
       <c r="B12">
-        <v>329</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46307.11458333334</v>
+        <v>46308.11458333334</v>
       </c>
       <c r="B13">
-        <v>327</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46307.125</v>
+        <v>46308.125</v>
       </c>
       <c r="B14">
-        <v>308</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46307.13541666666</v>
+        <v>46308.13541666666</v>
       </c>
       <c r="B15">
-        <v>303</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46307.14583333334</v>
+        <v>46308.14583333334</v>
       </c>
       <c r="B16">
-        <v>304</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46307.15625</v>
+        <v>46308.15625</v>
       </c>
       <c r="B17">
-        <v>304</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46307.16666666666</v>
+        <v>46308.16666666666</v>
       </c>
       <c r="B18">
-        <v>258</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46307.17708333334</v>
+        <v>46308.17708333334</v>
       </c>
       <c r="B19">
-        <v>261</v>
+        <v>182</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46307.1875</v>
+        <v>46308.1875</v>
       </c>
       <c r="B20">
-        <v>265</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46307.19791666666</v>
+        <v>46308.19791666666</v>
       </c>
       <c r="B21">
-        <v>266</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46307.20833333334</v>
+        <v>46308.20833333334</v>
       </c>
       <c r="B22">
-        <v>378</v>
+        <v>193</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46307.21875</v>
+        <v>46308.21875</v>
       </c>
       <c r="B23">
-        <v>390</v>
+        <v>193</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46307.22916666666</v>
+        <v>46308.22916666666</v>
       </c>
       <c r="B24">
-        <v>403</v>
+        <v>193</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46307.23958333334</v>
+        <v>46308.23958333334</v>
       </c>
       <c r="B25">
-        <v>412</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46307.25</v>
+        <v>46308.25</v>
       </c>
       <c r="B26">
-        <v>451</v>
+        <v>490</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46307.26041666666</v>
+        <v>46308.26041666666</v>
       </c>
       <c r="B27">
-        <v>459</v>
+        <v>514</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46307.27083333334</v>
+        <v>46308.27083333334</v>
       </c>
       <c r="B28">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46307.28125</v>
+        <v>46308.28125</v>
       </c>
       <c r="B29">
-        <v>480</v>
+        <v>516</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46307.29166666666</v>
+        <v>46308.29166666666</v>
       </c>
       <c r="B30">
-        <v>468</v>
+        <v>514</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46307.30208333334</v>
+        <v>46308.30208333334</v>
       </c>
       <c r="B31">
-        <v>514</v>
+        <v>526</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46307.3125</v>
+        <v>46308.3125</v>
       </c>
       <c r="B32">
-        <v>674</v>
+        <v>527</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46307.32291666666</v>
+        <v>46308.32291666666</v>
       </c>
       <c r="B33">
-        <v>678</v>
+        <v>526</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46307.33333333334</v>
+        <v>46308.33333333334</v>
       </c>
       <c r="B34">
-        <v>646</v>
+        <v>508</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46307.34375</v>
+        <v>46308.34375</v>
       </c>
       <c r="B35">
-        <v>650</v>
+        <v>498</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46307.35416666666</v>
+        <v>46308.35416666666</v>
       </c>
       <c r="B36">
-        <v>634</v>
+        <v>506</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46307.36458333334</v>
+        <v>46308.36458333334</v>
       </c>
       <c r="B37">
-        <v>638</v>
+        <v>503</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46307.375</v>
+        <v>46308.375</v>
       </c>
       <c r="B38">
-        <v>462</v>
+        <v>471</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46307.38541666666</v>
+        <v>46308.38541666666</v>
       </c>
       <c r="B39">
-        <v>440</v>
+        <v>468</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46307.39583333334</v>
+        <v>46308.39583333334</v>
       </c>
       <c r="B40">
-        <v>438</v>
+        <v>471</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46307.40625</v>
+        <v>46308.40625</v>
       </c>
       <c r="B41">
-        <v>425</v>
+        <v>465</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46307.41666666666</v>
+        <v>46308.41666666666</v>
       </c>
       <c r="B42">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46307.42708333334</v>
+        <v>46308.42708333334</v>
       </c>
       <c r="B43">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46307.4375</v>
+        <v>46308.4375</v>
       </c>
       <c r="B44">
-        <v>249</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46307.44791666666</v>
+        <v>46308.44791666666</v>
       </c>
       <c r="B45">
-        <v>206</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46307.45833333334</v>
+        <v>46308.45833333334</v>
       </c>
       <c r="B46">
-        <v>275</v>
+        <v>198</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46307.46875</v>
+        <v>46308.46875</v>
       </c>
       <c r="B47">
-        <v>286</v>
+        <v>199</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46307.47916666666</v>
+        <v>46308.47916666666</v>
       </c>
       <c r="B48">
-        <v>286</v>
+        <v>201</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46307.48958333334</v>
+        <v>46308.48958333334</v>
       </c>
       <c r="B49">
-        <v>286</v>
+        <v>199</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46307.5</v>
+        <v>46308.5</v>
       </c>
       <c r="B50">
-        <v>261</v>
+        <v>191</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46307.51041666666</v>
+        <v>46308.51041666666</v>
       </c>
       <c r="B51">
-        <v>261</v>
+        <v>194</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46307.52083333334</v>
+        <v>46308.52083333334</v>
       </c>
       <c r="B52">
-        <v>265</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46307.53125</v>
+        <v>46308.53125</v>
       </c>
       <c r="B53">
-        <v>260</v>
+        <v>166</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46307.54166666666</v>
+        <v>46308.54166666666</v>
       </c>
       <c r="B54">
-        <v>252</v>
+        <v>204</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46307.55208333334</v>
+        <v>46308.55208333334</v>
       </c>
       <c r="B55">
-        <v>214</v>
+        <v>204</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46307.5625</v>
+        <v>46308.5625</v>
       </c>
       <c r="B56">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46307.57291666666</v>
+        <v>46308.57291666666</v>
       </c>
       <c r="B57">
-        <v>212</v>
+        <v>204</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46307.58333333334</v>
+        <v>46308.58333333334</v>
       </c>
       <c r="B58">
-        <v>219</v>
+        <v>193</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46307.59375</v>
+        <v>46308.59375</v>
       </c>
       <c r="B59">
-        <v>221</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46307.60416666666</v>
+        <v>46308.60416666666</v>
       </c>
       <c r="B60">
-        <v>224</v>
+        <v>193</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46307.61458333334</v>
+        <v>46308.61458333334</v>
       </c>
       <c r="B61">
-        <v>222</v>
+        <v>193</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46307.625</v>
+        <v>46308.625</v>
       </c>
       <c r="B62">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46307.63541666666</v>
+        <v>46308.63541666666</v>
       </c>
       <c r="B63">
-        <v>210</v>
+        <v>227</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46307.64583333334</v>
+        <v>46308.64583333334</v>
       </c>
       <c r="B64">
-        <v>203</v>
+        <v>227</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46307.65625</v>
+        <v>46308.65625</v>
       </c>
       <c r="B65">
-        <v>210</v>
+        <v>243</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46307.66666666666</v>
+        <v>46308.66666666666</v>
       </c>
       <c r="B66">
-        <v>440</v>
+        <v>613</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46307.67708333334</v>
+        <v>46308.67708333334</v>
       </c>
       <c r="B67">
-        <v>459</v>
+        <v>638</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46307.6875</v>
+        <v>46308.6875</v>
       </c>
       <c r="B68">
-        <v>464</v>
+        <v>654</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46307.69791666666</v>
+        <v>46308.69791666666</v>
       </c>
       <c r="B69">
-        <v>483</v>
+        <v>658</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46307.70833333334</v>
+        <v>46308.70833333334</v>
       </c>
       <c r="B70">
-        <v>608</v>
+        <v>640</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46307.71875</v>
+        <v>46308.71875</v>
       </c>
       <c r="B71">
-        <v>618</v>
+        <v>675</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46307.72916666666</v>
+        <v>46308.72916666666</v>
       </c>
       <c r="B72">
-        <v>618</v>
+        <v>681</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46307.73958333334</v>
+        <v>46308.73958333334</v>
       </c>
       <c r="B73">
-        <v>648</v>
+        <v>684</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46307.75</v>
+        <v>46308.75</v>
       </c>
       <c r="B74">
-        <v>686</v>
+        <v>677</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46307.76041666666</v>
+        <v>46308.76041666666</v>
       </c>
       <c r="B75">
-        <v>698</v>
+        <v>678</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46307.77083333334</v>
+        <v>46308.77083333334</v>
       </c>
       <c r="B76">
-        <v>697</v>
+        <v>682</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46307.78125</v>
+        <v>46308.78125</v>
       </c>
       <c r="B77">
-        <v>699</v>
+        <v>679</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46307.79166666666</v>
+        <v>46308.79166666666</v>
       </c>
       <c r="B78">
-        <v>677</v>
+        <v>685</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46307.80208333334</v>
+        <v>46308.80208333334</v>
       </c>
       <c r="B79">
-        <v>675</v>
+        <v>685</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46307.8125</v>
+        <v>46308.8125</v>
       </c>
       <c r="B80">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46307.82291666666</v>
+        <v>46308.82291666666</v>
       </c>
       <c r="B81">
-        <v>685</v>
+        <v>649</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46307.83333333334</v>
+        <v>46308.83333333334</v>
       </c>
       <c r="B82">
-        <v>669</v>
+        <v>642</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46307.84375</v>
+        <v>46308.84375</v>
       </c>
       <c r="B83">
-        <v>627</v>
+        <v>638</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46307.85416666666</v>
+        <v>46308.85416666666</v>
       </c>
       <c r="B84">
-        <v>626</v>
+        <v>638</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46307.86458333334</v>
+        <v>46308.86458333334</v>
       </c>
       <c r="B85">
-        <v>606</v>
+        <v>637</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46307.875</v>
+        <v>46308.875</v>
       </c>
       <c r="B86">
-        <v>587</v>
+        <v>640</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46307.88541666666</v>
+        <v>46308.88541666666</v>
       </c>
       <c r="B87">
-        <v>593</v>
+        <v>636</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46307.89583333334</v>
+        <v>46308.89583333334</v>
       </c>
       <c r="B88">
-        <v>587</v>
+        <v>637</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46307.90625</v>
+        <v>46308.90625</v>
       </c>
       <c r="B89">
-        <v>576</v>
+        <v>636</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46307.91666666666</v>
+        <v>46308.91666666666</v>
       </c>
       <c r="B90">
-        <v>532</v>
+        <v>624</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46307.92708333334</v>
+        <v>46308.92708333334</v>
       </c>
       <c r="B91">
-        <v>525</v>
+        <v>636</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46307.9375</v>
+        <v>46308.9375</v>
       </c>
       <c r="B92">
-        <v>527</v>
+        <v>637</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46307.94791666666</v>
+        <v>46308.94791666666</v>
       </c>
       <c r="B93">
-        <v>524</v>
+        <v>652</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46307.95833333334</v>
+        <v>46308.95833333334</v>
       </c>
       <c r="B94">
-        <v>392</v>
+        <v>364</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46307.96875</v>
+        <v>46308.96875</v>
       </c>
       <c r="B95">
-        <v>386</v>
+        <v>342</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46307.97916666666</v>
+        <v>46308.97916666666</v>
       </c>
       <c r="B96">
-        <v>408</v>
+        <v>341</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46307.98958333334</v>
+        <v>46308.98958333334</v>
       </c>
       <c r="B97">
-        <v>434</v>
+        <v>346</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B98">
-        <v>289</v>
+        <v>417</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46308.01041666666</v>
+        <v>46309.01041666666</v>
       </c>
       <c r="B99">
-        <v>282</v>
+        <v>418</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46308.02083333334</v>
+        <v>46309.02083333334</v>
       </c>
       <c r="B100">
-        <v>282</v>
+        <v>417</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46308.03125</v>
+        <v>46309.03125</v>
       </c>
       <c r="B101">
-        <v>281</v>
+        <v>416</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46308.04166666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="B102">
-        <v>230</v>
+        <v>416</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46308.05208333334</v>
+        <v>46309.05208333334</v>
       </c>
       <c r="B103">
-        <v>225</v>
+        <v>414</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46308.0625</v>
+        <v>46309.0625</v>
       </c>
       <c r="B104">
-        <v>225</v>
+        <v>415</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46308.07291666666</v>
+        <v>46309.07291666666</v>
       </c>
       <c r="B105">
-        <v>225</v>
+        <v>415</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46308.08333333334</v>
+        <v>46309.08333333334</v>
       </c>
       <c r="B106">
-        <v>240</v>
+        <v>415</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46308.09375</v>
+        <v>46309.09375</v>
       </c>
       <c r="B107">
-        <v>241</v>
+        <v>415</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46308.10416666666</v>
+        <v>46309.10416666666</v>
       </c>
       <c r="B108">
-        <v>241</v>
+        <v>415</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46308.11458333334</v>
+        <v>46309.11458333334</v>
       </c>
       <c r="B109">
-        <v>239</v>
+        <v>415</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46308.125</v>
+        <v>46309.125</v>
       </c>
       <c r="B110">
-        <v>166</v>
+        <v>377</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46308.13541666666</v>
+        <v>46309.13541666666</v>
       </c>
       <c r="B111">
-        <v>164</v>
+        <v>374</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46308.14583333334</v>
+        <v>46309.14583333334</v>
       </c>
       <c r="B112">
-        <v>164</v>
+        <v>374</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46308.15625</v>
+        <v>46309.15625</v>
       </c>
       <c r="B113">
-        <v>164</v>
+        <v>375</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46308.16666666666</v>
+        <v>46309.16666666666</v>
       </c>
       <c r="B114">
-        <v>181</v>
+        <v>375</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46308.17708333334</v>
+        <v>46309.17708333334</v>
       </c>
       <c r="B115">
-        <v>182</v>
+        <v>375</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46308.1875</v>
+        <v>46309.1875</v>
       </c>
       <c r="B116">
-        <v>182</v>
+        <v>375</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46308.19791666666</v>
+        <v>46309.19791666666</v>
       </c>
       <c r="B117">
-        <v>182</v>
+        <v>377</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46308.20833333334</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="B118">
-        <v>193</v>
+        <v>441</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46308.21875</v>
+        <v>46309.21875</v>
       </c>
       <c r="B119">
-        <v>193</v>
+        <v>454</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46308.22916666666</v>
+        <v>46309.22916666666</v>
       </c>
       <c r="B120">
-        <v>193</v>
+        <v>491</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46308.23958333334</v>
+        <v>46309.23958333334</v>
       </c>
       <c r="B121">
-        <v>200</v>
+        <v>495</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46308.25</v>
+        <v>46309.25</v>
       </c>
       <c r="B122">
-        <v>490</v>
+        <v>522</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46308.26041666666</v>
+        <v>46309.26041666666</v>
       </c>
       <c r="B123">
-        <v>514</v>
+        <v>523</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46308.27083333334</v>
+        <v>46309.27083333334</v>
       </c>
       <c r="B124">
-        <v>513</v>
+        <v>525</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46308.28125</v>
+        <v>46309.28125</v>
       </c>
       <c r="B125">
-        <v>516</v>
+        <v>526</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46308.29166666666</v>
+        <v>46309.29166666666</v>
       </c>
       <c r="B126">
-        <v>514</v>
+        <v>536</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46308.30208333334</v>
+        <v>46309.30208333334</v>
       </c>
       <c r="B127">
-        <v>526</v>
+        <v>535</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46308.3125</v>
+        <v>46309.3125</v>
       </c>
       <c r="B128">
-        <v>527</v>
+        <v>539</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46308.32291666666</v>
+        <v>46309.32291666666</v>
       </c>
       <c r="B129">
-        <v>526</v>
+        <v>505</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46308.33333333334</v>
+        <v>46309.33333333334</v>
       </c>
       <c r="B130">
-        <v>508</v>
+        <v>494</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46308.34375</v>
+        <v>46309.34375</v>
       </c>
       <c r="B131">
-        <v>498</v>
+        <v>486</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46308.35416666666</v>
+        <v>46309.35416666666</v>
       </c>
       <c r="B132">
-        <v>506</v>
+        <v>480</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46308.36458333334</v>
+        <v>46309.36458333334</v>
       </c>
       <c r="B133">
-        <v>503</v>
+        <v>483</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46308.375</v>
+        <v>46309.375</v>
       </c>
       <c r="B134">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46308.38541666666</v>
+        <v>46309.38541666666</v>
       </c>
       <c r="B135">
         <v>468</v>
@@ -1466,122 +1466,162 @@
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46308.39583333334</v>
+        <v>46309.39583333334</v>
       </c>
       <c r="B136">
-        <v>471</v>
+        <v>486</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46308.40625</v>
+        <v>46309.40625</v>
       </c>
       <c r="B137">
-        <v>465</v>
+        <v>484</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46308.41666666666</v>
+        <v>46309.41666666666</v>
       </c>
       <c r="B138">
-        <v>215</v>
+        <v>440</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46308.42708333334</v>
+        <v>46309.42708333334</v>
       </c>
       <c r="B139">
-        <v>191</v>
+        <v>437</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46308.4375</v>
+        <v>46309.4375</v>
       </c>
       <c r="B140">
-        <v>195</v>
+        <v>426</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46308.44791666666</v>
+        <v>46309.44791666666</v>
       </c>
       <c r="B141">
-        <v>189</v>
+        <v>417</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46308.45833333334</v>
+        <v>46309.45833333334</v>
       </c>
       <c r="B142">
-        <v>198</v>
+        <v>427</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46308.46875</v>
+        <v>46309.46875</v>
       </c>
       <c r="B143">
-        <v>199</v>
+        <v>429</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46308.47916666666</v>
+        <v>46309.47916666666</v>
       </c>
       <c r="B144">
-        <v>201</v>
+        <v>437</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46308.48958333334</v>
+        <v>46309.48958333334</v>
       </c>
       <c r="B145">
-        <v>199</v>
+        <v>459</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46308.5</v>
+        <v>46309.5</v>
       </c>
       <c r="B146">
-        <v>191</v>
+        <v>455</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="2">
-        <v>46308.51041666666</v>
+        <v>46309.51041666666</v>
       </c>
       <c r="B147">
-        <v>194</v>
+        <v>453</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="2">
-        <v>46308.52083333334</v>
+        <v>46309.52083333334</v>
       </c>
       <c r="B148">
-        <v>168</v>
+        <v>448</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="2">
-        <v>46308.53125</v>
+        <v>46309.53125</v>
       </c>
       <c r="B149">
-        <v>166</v>
+        <v>379</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" s="2">
-        <v>46308.54166666666</v>
+        <v>46309.54166666666</v>
       </c>
       <c r="B150">
-        <v>204</v>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="2">
+        <v>46309.55208333334</v>
+      </c>
+      <c r="B151">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="2">
+        <v>46309.5625</v>
+      </c>
+      <c r="B152">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="2">
+        <v>46309.57291666666</v>
+      </c>
+      <c r="B153">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="2">
+        <v>46309.58333333334</v>
+      </c>
+      <c r="B154">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="2">
+        <v>46309.59375</v>
+      </c>
+      <c r="B155">
+        <v>330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for GESS
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B155"/>
+  <dimension ref="A1:B146"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,631 +394,631 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B2">
-        <v>289</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46308.01041666666</v>
+        <v>46310.01041666666</v>
       </c>
       <c r="B3">
-        <v>282</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46308.02083333334</v>
+        <v>46310.02083333334</v>
       </c>
       <c r="B4">
-        <v>282</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46308.03125</v>
+        <v>46310.03125</v>
       </c>
       <c r="B5">
-        <v>281</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46308.04166666666</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="B6">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46308.05208333334</v>
+        <v>46310.05208333334</v>
       </c>
       <c r="B7">
-        <v>225</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46308.0625</v>
+        <v>46310.0625</v>
       </c>
       <c r="B8">
-        <v>225</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46308.07291666666</v>
+        <v>46310.07291666666</v>
       </c>
       <c r="B9">
-        <v>225</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46308.08333333334</v>
+        <v>46310.08333333334</v>
       </c>
       <c r="B10">
-        <v>240</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46308.09375</v>
+        <v>46310.09375</v>
       </c>
       <c r="B11">
-        <v>241</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46308.10416666666</v>
+        <v>46310.10416666666</v>
       </c>
       <c r="B12">
-        <v>241</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46308.11458333334</v>
+        <v>46310.11458333334</v>
       </c>
       <c r="B13">
-        <v>239</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46308.125</v>
+        <v>46310.125</v>
       </c>
       <c r="B14">
-        <v>166</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46308.13541666666</v>
+        <v>46310.13541666666</v>
       </c>
       <c r="B15">
-        <v>164</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46308.14583333334</v>
+        <v>46310.14583333334</v>
       </c>
       <c r="B16">
-        <v>164</v>
+        <v>207</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46308.15625</v>
+        <v>46310.15625</v>
       </c>
       <c r="B17">
-        <v>164</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46308.16666666666</v>
+        <v>46310.16666666666</v>
       </c>
       <c r="B18">
-        <v>181</v>
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46308.17708333334</v>
+        <v>46310.17708333334</v>
       </c>
       <c r="B19">
-        <v>182</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46308.1875</v>
+        <v>46310.1875</v>
       </c>
       <c r="B20">
-        <v>182</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46308.19791666666</v>
+        <v>46310.19791666666</v>
       </c>
       <c r="B21">
-        <v>182</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46308.20833333334</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="B22">
-        <v>193</v>
+        <v>366</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46308.21875</v>
+        <v>46310.21875</v>
       </c>
       <c r="B23">
-        <v>193</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46308.22916666666</v>
+        <v>46310.22916666666</v>
       </c>
       <c r="B24">
-        <v>193</v>
+        <v>385</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46308.23958333334</v>
+        <v>46310.23958333334</v>
       </c>
       <c r="B25">
-        <v>200</v>
+        <v>389</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46308.25</v>
+        <v>46310.25</v>
       </c>
       <c r="B26">
-        <v>490</v>
+        <v>516</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46308.26041666666</v>
+        <v>46310.26041666666</v>
       </c>
       <c r="B27">
-        <v>514</v>
+        <v>517</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46308.27083333334</v>
+        <v>46310.27083333334</v>
       </c>
       <c r="B28">
-        <v>513</v>
+        <v>533</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46308.28125</v>
+        <v>46310.28125</v>
       </c>
       <c r="B29">
-        <v>516</v>
+        <v>589</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46308.29166666666</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="B30">
-        <v>514</v>
+        <v>555</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46308.30208333334</v>
+        <v>46310.30208333334</v>
       </c>
       <c r="B31">
-        <v>526</v>
+        <v>565</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46308.3125</v>
+        <v>46310.3125</v>
       </c>
       <c r="B32">
-        <v>527</v>
+        <v>586</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46308.32291666666</v>
+        <v>46310.32291666666</v>
       </c>
       <c r="B33">
-        <v>526</v>
+        <v>598</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46308.33333333334</v>
+        <v>46310.33333333334</v>
       </c>
       <c r="B34">
-        <v>508</v>
+        <v>541</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46308.34375</v>
+        <v>46310.34375</v>
       </c>
       <c r="B35">
-        <v>498</v>
+        <v>552</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46308.35416666666</v>
+        <v>46310.35416666666</v>
       </c>
       <c r="B36">
-        <v>506</v>
+        <v>710</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46308.36458333334</v>
+        <v>46310.36458333334</v>
       </c>
       <c r="B37">
-        <v>503</v>
+        <v>749</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46308.375</v>
+        <v>46310.375</v>
       </c>
       <c r="B38">
-        <v>471</v>
+        <v>581</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46308.38541666666</v>
+        <v>46310.38541666666</v>
       </c>
       <c r="B39">
-        <v>468</v>
+        <v>561</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46308.39583333334</v>
+        <v>46310.39583333334</v>
       </c>
       <c r="B40">
-        <v>471</v>
+        <v>561</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46308.40625</v>
+        <v>46310.40625</v>
       </c>
       <c r="B41">
-        <v>465</v>
+        <v>555</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46308.41666666666</v>
+        <v>46310.41666666666</v>
       </c>
       <c r="B42">
-        <v>215</v>
+        <v>324</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46308.42708333334</v>
+        <v>46310.42708333334</v>
       </c>
       <c r="B43">
-        <v>191</v>
+        <v>304</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46308.4375</v>
+        <v>46310.4375</v>
       </c>
       <c r="B44">
-        <v>195</v>
+        <v>305</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46308.44791666666</v>
+        <v>46310.44791666666</v>
       </c>
       <c r="B45">
-        <v>189</v>
+        <v>303</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46308.45833333334</v>
+        <v>46310.45833333334</v>
       </c>
       <c r="B46">
-        <v>198</v>
+        <v>312</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46308.46875</v>
+        <v>46310.46875</v>
       </c>
       <c r="B47">
-        <v>199</v>
+        <v>323</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46308.47916666666</v>
+        <v>46310.47916666666</v>
       </c>
       <c r="B48">
-        <v>201</v>
+        <v>300</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46308.48958333334</v>
+        <v>46310.48958333334</v>
       </c>
       <c r="B49">
-        <v>199</v>
+        <v>295</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46308.5</v>
+        <v>46310.5</v>
       </c>
       <c r="B50">
-        <v>191</v>
+        <v>276</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46308.51041666666</v>
+        <v>46310.51041666666</v>
       </c>
       <c r="B51">
-        <v>194</v>
+        <v>249</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46308.52083333334</v>
+        <v>46310.52083333334</v>
       </c>
       <c r="B52">
-        <v>168</v>
+        <v>230</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46308.53125</v>
+        <v>46310.53125</v>
       </c>
       <c r="B53">
-        <v>166</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46308.54166666666</v>
+        <v>46310.54166666666</v>
       </c>
       <c r="B54">
-        <v>204</v>
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46308.55208333334</v>
+        <v>46310.55208333334</v>
       </c>
       <c r="B55">
-        <v>204</v>
+        <v>248</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46308.5625</v>
+        <v>46310.5625</v>
       </c>
       <c r="B56">
-        <v>204</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46308.57291666666</v>
+        <v>46310.57291666666</v>
       </c>
       <c r="B57">
-        <v>204</v>
+        <v>238</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46308.58333333334</v>
+        <v>46310.58333333334</v>
       </c>
       <c r="B58">
-        <v>193</v>
+        <v>224</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46308.59375</v>
+        <v>46310.59375</v>
       </c>
       <c r="B59">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46308.60416666666</v>
+        <v>46310.60416666666</v>
       </c>
       <c r="B60">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46308.61458333334</v>
+        <v>46310.61458333334</v>
       </c>
       <c r="B61">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46308.625</v>
+        <v>46310.625</v>
       </c>
       <c r="B62">
-        <v>215</v>
+        <v>226</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46308.63541666666</v>
+        <v>46310.63541666666</v>
       </c>
       <c r="B63">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46308.64583333334</v>
+        <v>46310.64583333334</v>
       </c>
       <c r="B64">
-        <v>227</v>
+        <v>209</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46308.65625</v>
+        <v>46310.65625</v>
       </c>
       <c r="B65">
-        <v>243</v>
+        <v>259</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46308.66666666666</v>
+        <v>46310.66666666666</v>
       </c>
       <c r="B66">
-        <v>613</v>
+        <v>603</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46308.67708333334</v>
+        <v>46310.67708333334</v>
       </c>
       <c r="B67">
-        <v>638</v>
+        <v>652</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46308.6875</v>
+        <v>46310.6875</v>
       </c>
       <c r="B68">
-        <v>654</v>
+        <v>632</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46308.69791666666</v>
+        <v>46310.69791666666</v>
       </c>
       <c r="B69">
-        <v>658</v>
+        <v>633</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46308.70833333334</v>
+        <v>46310.70833333334</v>
       </c>
       <c r="B70">
-        <v>640</v>
+        <v>663</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46308.71875</v>
+        <v>46310.71875</v>
       </c>
       <c r="B71">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46308.72916666666</v>
+        <v>46310.72916666666</v>
       </c>
       <c r="B72">
-        <v>681</v>
+        <v>672</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46308.73958333334</v>
+        <v>46310.73958333334</v>
       </c>
       <c r="B73">
-        <v>684</v>
+        <v>710</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46308.75</v>
+        <v>46310.75</v>
       </c>
       <c r="B74">
-        <v>677</v>
+        <v>689</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46308.76041666666</v>
+        <v>46310.76041666666</v>
       </c>
       <c r="B75">
-        <v>678</v>
+        <v>692</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46308.77083333334</v>
+        <v>46310.77083333334</v>
       </c>
       <c r="B76">
-        <v>682</v>
+        <v>678</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46308.78125</v>
+        <v>46310.78125</v>
       </c>
       <c r="B77">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46308.79166666666</v>
+        <v>46310.79166666666</v>
       </c>
       <c r="B78">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46308.80208333334</v>
+        <v>46310.80208333334</v>
       </c>
       <c r="B79">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46308.8125</v>
+        <v>46310.8125</v>
       </c>
       <c r="B80">
         <v>687</v>
@@ -1026,63 +1026,63 @@
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46308.82291666666</v>
+        <v>46310.82291666666</v>
       </c>
       <c r="B81">
-        <v>649</v>
+        <v>688</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46308.83333333334</v>
+        <v>46310.83333333334</v>
       </c>
       <c r="B82">
-        <v>642</v>
+        <v>682</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46308.84375</v>
+        <v>46310.84375</v>
       </c>
       <c r="B83">
-        <v>638</v>
+        <v>677</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46308.85416666666</v>
+        <v>46310.85416666666</v>
       </c>
       <c r="B84">
-        <v>638</v>
+        <v>677</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46308.86458333334</v>
+        <v>46310.86458333334</v>
       </c>
       <c r="B85">
-        <v>637</v>
+        <v>658</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46308.875</v>
+        <v>46310.875</v>
       </c>
       <c r="B86">
-        <v>640</v>
+        <v>638</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46308.88541666666</v>
+        <v>46310.88541666666</v>
       </c>
       <c r="B87">
-        <v>636</v>
+        <v>637</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46308.89583333334</v>
+        <v>46310.89583333334</v>
       </c>
       <c r="B88">
         <v>637</v>
@@ -1090,95 +1090,95 @@
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46308.90625</v>
+        <v>46310.90625</v>
       </c>
       <c r="B89">
-        <v>636</v>
+        <v>650</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46308.91666666666</v>
+        <v>46310.91666666666</v>
       </c>
       <c r="B90">
-        <v>624</v>
+        <v>550</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46308.92708333334</v>
+        <v>46310.92708333334</v>
       </c>
       <c r="B91">
-        <v>636</v>
+        <v>527</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46308.9375</v>
+        <v>46310.9375</v>
       </c>
       <c r="B92">
-        <v>637</v>
+        <v>527</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46308.94791666666</v>
+        <v>46310.94791666666</v>
       </c>
       <c r="B93">
-        <v>652</v>
+        <v>525</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46308.95833333334</v>
+        <v>46310.95833333334</v>
       </c>
       <c r="B94">
-        <v>364</v>
+        <v>452</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46308.96875</v>
+        <v>46310.96875</v>
       </c>
       <c r="B95">
-        <v>342</v>
+        <v>441</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46308.97916666666</v>
+        <v>46310.97916666666</v>
       </c>
       <c r="B96">
-        <v>341</v>
+        <v>441</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46308.98958333334</v>
+        <v>46310.98958333334</v>
       </c>
       <c r="B97">
-        <v>346</v>
+        <v>439</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="B98">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46309.01041666666</v>
+        <v>46311.01041666666</v>
       </c>
       <c r="B99">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46309.02083333334</v>
+        <v>46311.02083333334</v>
       </c>
       <c r="B100">
         <v>417</v>
@@ -1186,442 +1186,370 @@
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46309.03125</v>
+        <v>46311.03125</v>
       </c>
       <c r="B101">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46309.04166666666</v>
+        <v>46311.04166666666</v>
       </c>
       <c r="B102">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46309.05208333334</v>
+        <v>46311.05208333334</v>
       </c>
       <c r="B103">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46309.0625</v>
+        <v>46311.0625</v>
       </c>
       <c r="B104">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46309.07291666666</v>
+        <v>46311.07291666666</v>
       </c>
       <c r="B105">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46309.08333333334</v>
+        <v>46311.08333333334</v>
       </c>
       <c r="B106">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46309.09375</v>
+        <v>46311.09375</v>
       </c>
       <c r="B107">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46309.10416666666</v>
+        <v>46311.10416666666</v>
       </c>
       <c r="B108">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46309.11458333334</v>
+        <v>46311.11458333334</v>
       </c>
       <c r="B109">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46309.125</v>
+        <v>46311.125</v>
       </c>
       <c r="B110">
-        <v>377</v>
+        <v>403</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46309.13541666666</v>
+        <v>46311.13541666666</v>
       </c>
       <c r="B111">
-        <v>374</v>
+        <v>403</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46309.14583333334</v>
+        <v>46311.14583333334</v>
       </c>
       <c r="B112">
-        <v>374</v>
+        <v>403</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46309.15625</v>
+        <v>46311.15625</v>
       </c>
       <c r="B113">
-        <v>375</v>
+        <v>402</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46309.16666666666</v>
+        <v>46311.16666666666</v>
       </c>
       <c r="B114">
-        <v>375</v>
+        <v>403</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46309.17708333334</v>
+        <v>46311.17708333334</v>
       </c>
       <c r="B115">
-        <v>375</v>
+        <v>403</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46309.1875</v>
+        <v>46311.1875</v>
       </c>
       <c r="B116">
-        <v>375</v>
+        <v>403</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46309.19791666666</v>
+        <v>46311.19791666666</v>
       </c>
       <c r="B117">
-        <v>377</v>
+        <v>402</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46309.20833333334</v>
+        <v>46311.20833333334</v>
       </c>
       <c r="B118">
-        <v>441</v>
+        <v>417</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46309.21875</v>
+        <v>46311.21875</v>
       </c>
       <c r="B119">
-        <v>454</v>
+        <v>420</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46309.22916666666</v>
+        <v>46311.22916666666</v>
       </c>
       <c r="B120">
-        <v>491</v>
+        <v>421</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46309.23958333334</v>
+        <v>46311.23958333334</v>
       </c>
       <c r="B121">
-        <v>495</v>
+        <v>421</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46309.25</v>
+        <v>46311.25</v>
       </c>
       <c r="B122">
-        <v>522</v>
+        <v>416</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46309.26041666666</v>
+        <v>46311.26041666666</v>
       </c>
       <c r="B123">
-        <v>523</v>
+        <v>411</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46309.27083333334</v>
+        <v>46311.27083333334</v>
       </c>
       <c r="B124">
-        <v>525</v>
+        <v>414</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46309.28125</v>
+        <v>46311.28125</v>
       </c>
       <c r="B125">
-        <v>526</v>
+        <v>415</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46309.29166666666</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="B126">
-        <v>536</v>
+        <v>449</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46309.30208333334</v>
+        <v>46311.30208333334</v>
       </c>
       <c r="B127">
-        <v>535</v>
+        <v>448</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46309.3125</v>
+        <v>46311.3125</v>
       </c>
       <c r="B128">
-        <v>539</v>
+        <v>458</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46309.32291666666</v>
+        <v>46311.32291666666</v>
       </c>
       <c r="B129">
-        <v>505</v>
+        <v>459</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46309.33333333334</v>
+        <v>46311.33333333334</v>
       </c>
       <c r="B130">
-        <v>494</v>
+        <v>446</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46309.34375</v>
+        <v>46311.34375</v>
       </c>
       <c r="B131">
-        <v>486</v>
+        <v>443</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46309.35416666666</v>
+        <v>46311.35416666666</v>
       </c>
       <c r="B132">
-        <v>480</v>
+        <v>445</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="2">
-        <v>46309.36458333334</v>
+        <v>46311.36458333334</v>
       </c>
       <c r="B133">
-        <v>483</v>
+        <v>457</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="2">
-        <v>46309.375</v>
+        <v>46311.375</v>
       </c>
       <c r="B134">
-        <v>470</v>
+        <v>440</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="2">
-        <v>46309.38541666666</v>
+        <v>46311.38541666666</v>
       </c>
       <c r="B135">
-        <v>468</v>
+        <v>440</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="2">
-        <v>46309.39583333334</v>
+        <v>46311.39583333334</v>
       </c>
       <c r="B136">
-        <v>486</v>
+        <v>438</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="2">
-        <v>46309.40625</v>
+        <v>46311.40625</v>
       </c>
       <c r="B137">
-        <v>484</v>
+        <v>438</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="2">
-        <v>46309.41666666666</v>
+        <v>46311.41666666666</v>
       </c>
       <c r="B138">
-        <v>440</v>
+        <v>184</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="2">
-        <v>46309.42708333334</v>
+        <v>46311.42708333334</v>
       </c>
       <c r="B139">
-        <v>437</v>
+        <v>208</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="2">
-        <v>46309.4375</v>
+        <v>46311.4375</v>
       </c>
       <c r="B140">
-        <v>426</v>
+        <v>207</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="2">
-        <v>46309.44791666666</v>
+        <v>46311.44791666666</v>
       </c>
       <c r="B141">
-        <v>417</v>
+        <v>207</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="2">
-        <v>46309.45833333334</v>
+        <v>46311.45833333334</v>
       </c>
       <c r="B142">
-        <v>427</v>
+        <v>214</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="2">
-        <v>46309.46875</v>
+        <v>46311.46875</v>
       </c>
       <c r="B143">
-        <v>429</v>
+        <v>216</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="2">
-        <v>46309.47916666666</v>
+        <v>46311.47916666666</v>
       </c>
       <c r="B144">
-        <v>437</v>
+        <v>217</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" s="2">
-        <v>46309.48958333334</v>
+        <v>46311.48958333334</v>
       </c>
       <c r="B145">
-        <v>459</v>
+        <v>215</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="2">
-        <v>46309.5</v>
+        <v>46311.5</v>
       </c>
       <c r="B146">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2">
-      <c r="A147" s="2">
-        <v>46309.51041666666</v>
-      </c>
-      <c r="B147">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2">
-      <c r="A148" s="2">
-        <v>46309.52083333334</v>
-      </c>
-      <c r="B148">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2">
-      <c r="A149" s="2">
-        <v>46309.53125</v>
-      </c>
-      <c r="B149">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2">
-      <c r="A150" s="2">
-        <v>46309.54166666666</v>
-      </c>
-      <c r="B150">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2">
-      <c r="A151" s="2">
-        <v>46309.55208333334</v>
-      </c>
-      <c r="B151">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2">
-      <c r="A152" s="2">
-        <v>46309.5625</v>
-      </c>
-      <c r="B152">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2">
-      <c r="A153" s="2">
-        <v>46309.57291666666</v>
-      </c>
-      <c r="B153">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2">
-      <c r="A154" s="2">
-        <v>46309.58333333334</v>
-      </c>
-      <c r="B154">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2">
-      <c r="A155" s="2">
-        <v>46309.59375</v>
-      </c>
-      <c r="B155">
-        <v>330</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating model for Imperial
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Hydro_River.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B146"/>
+  <dimension ref="A1:B132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,495 +394,495 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="B2">
-        <v>238</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46310.01041666666</v>
+        <v>46315.01041666666</v>
       </c>
       <c r="B3">
-        <v>223</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46310.02083333334</v>
+        <v>46315.02083333334</v>
       </c>
       <c r="B4">
-        <v>224</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46310.03125</v>
+        <v>46315.03125</v>
       </c>
       <c r="B5">
-        <v>224</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46310.04166666666</v>
+        <v>46315.04166666666</v>
       </c>
       <c r="B6">
-        <v>228</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46310.05208333334</v>
+        <v>46315.05208333334</v>
       </c>
       <c r="B7">
-        <v>208</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46310.0625</v>
+        <v>46315.0625</v>
       </c>
       <c r="B8">
-        <v>207</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46310.07291666666</v>
+        <v>46315.07291666666</v>
       </c>
       <c r="B9">
-        <v>207</v>
+        <v>321</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46310.08333333334</v>
+        <v>46315.08333333334</v>
       </c>
       <c r="B10">
-        <v>207</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46310.09375</v>
+        <v>46315.09375</v>
       </c>
       <c r="B11">
-        <v>207</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46310.10416666666</v>
+        <v>46315.10416666666</v>
       </c>
       <c r="B12">
-        <v>207</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46310.11458333334</v>
+        <v>46315.11458333334</v>
       </c>
       <c r="B13">
-        <v>207</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46310.125</v>
+        <v>46315.125</v>
       </c>
       <c r="B14">
-        <v>207</v>
+        <v>243</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46310.13541666666</v>
+        <v>46315.13541666666</v>
       </c>
       <c r="B15">
-        <v>207</v>
+        <v>243</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46310.14583333334</v>
+        <v>46315.14583333334</v>
       </c>
       <c r="B16">
-        <v>207</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46310.15625</v>
+        <v>46315.15625</v>
       </c>
       <c r="B17">
-        <v>207</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46310.16666666666</v>
+        <v>46315.16666666666</v>
       </c>
       <c r="B18">
-        <v>207</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46310.17708333334</v>
+        <v>46315.17708333334</v>
       </c>
       <c r="B19">
-        <v>207</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46310.1875</v>
+        <v>46315.1875</v>
       </c>
       <c r="B20">
-        <v>207</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46310.19791666666</v>
+        <v>46315.19791666666</v>
       </c>
       <c r="B21">
-        <v>207</v>
+        <v>294</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46310.20833333334</v>
+        <v>46315.20833333334</v>
       </c>
       <c r="B22">
-        <v>366</v>
+        <v>401</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46310.21875</v>
+        <v>46315.21875</v>
       </c>
       <c r="B23">
-        <v>384</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46310.22916666666</v>
+        <v>46315.22916666666</v>
       </c>
       <c r="B24">
-        <v>385</v>
+        <v>415</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46310.23958333334</v>
+        <v>46315.23958333334</v>
       </c>
       <c r="B25">
-        <v>389</v>
+        <v>417</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46310.25</v>
+        <v>46315.25</v>
       </c>
       <c r="B26">
-        <v>516</v>
+        <v>522</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46310.26041666666</v>
+        <v>46315.26041666666</v>
       </c>
       <c r="B27">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46310.27083333334</v>
+        <v>46315.27083333334</v>
       </c>
       <c r="B28">
-        <v>533</v>
+        <v>527</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46310.28125</v>
+        <v>46315.28125</v>
       </c>
       <c r="B29">
-        <v>589</v>
+        <v>528</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46310.29166666666</v>
+        <v>46315.29166666666</v>
       </c>
       <c r="B30">
-        <v>555</v>
+        <v>566</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46310.30208333334</v>
+        <v>46315.30208333334</v>
       </c>
       <c r="B31">
-        <v>565</v>
+        <v>560</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46310.3125</v>
+        <v>46315.3125</v>
       </c>
       <c r="B32">
-        <v>586</v>
+        <v>560</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46310.32291666666</v>
+        <v>46315.32291666666</v>
       </c>
       <c r="B33">
-        <v>598</v>
+        <v>562</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46310.33333333334</v>
+        <v>46315.33333333334</v>
       </c>
       <c r="B34">
-        <v>541</v>
+        <v>509</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46310.34375</v>
+        <v>46315.34375</v>
       </c>
       <c r="B35">
-        <v>552</v>
+        <v>504</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46310.35416666666</v>
+        <v>46315.35416666666</v>
       </c>
       <c r="B36">
-        <v>710</v>
+        <v>515</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46310.36458333334</v>
+        <v>46315.36458333334</v>
       </c>
       <c r="B37">
-        <v>749</v>
+        <v>517</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46310.375</v>
+        <v>46315.375</v>
       </c>
       <c r="B38">
-        <v>581</v>
+        <v>519</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46310.38541666666</v>
+        <v>46315.38541666666</v>
       </c>
       <c r="B39">
-        <v>561</v>
+        <v>524</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46310.39583333334</v>
+        <v>46315.39583333334</v>
       </c>
       <c r="B40">
-        <v>561</v>
+        <v>518</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2">
-        <v>46310.40625</v>
+        <v>46315.40625</v>
       </c>
       <c r="B41">
-        <v>555</v>
+        <v>518</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2">
-        <v>46310.41666666666</v>
+        <v>46315.41666666666</v>
       </c>
       <c r="B42">
-        <v>324</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2">
-        <v>46310.42708333334</v>
+        <v>46315.42708333334</v>
       </c>
       <c r="B43">
-        <v>304</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2">
-        <v>46310.4375</v>
+        <v>46315.4375</v>
       </c>
       <c r="B44">
-        <v>305</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="2">
-        <v>46310.44791666666</v>
+        <v>46315.44791666666</v>
       </c>
       <c r="B45">
-        <v>303</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="2">
-        <v>46310.45833333334</v>
+        <v>46315.45833333334</v>
       </c>
       <c r="B46">
-        <v>312</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="2">
-        <v>46310.46875</v>
+        <v>46315.46875</v>
       </c>
       <c r="B47">
-        <v>323</v>
+        <v>207</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="2">
-        <v>46310.47916666666</v>
+        <v>46315.47916666666</v>
       </c>
       <c r="B48">
-        <v>300</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2">
-        <v>46310.48958333334</v>
+        <v>46315.48958333334</v>
       </c>
       <c r="B49">
-        <v>295</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="2">
-        <v>46310.5</v>
+        <v>46315.5</v>
       </c>
       <c r="B50">
-        <v>276</v>
+        <v>197</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="2">
-        <v>46310.51041666666</v>
+        <v>46315.51041666666</v>
       </c>
       <c r="B51">
-        <v>249</v>
+        <v>212</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="2">
-        <v>46310.52083333334</v>
+        <v>46315.52083333334</v>
       </c>
       <c r="B52">
-        <v>230</v>
+        <v>196</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="2">
-        <v>46310.53125</v>
+        <v>46315.53125</v>
       </c>
       <c r="B53">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="2">
-        <v>46310.54166666666</v>
+        <v>46315.54166666666</v>
       </c>
       <c r="B54">
-        <v>245</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="2">
-        <v>46310.55208333334</v>
+        <v>46315.55208333334</v>
       </c>
       <c r="B55">
-        <v>248</v>
+        <v>235</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="2">
-        <v>46310.5625</v>
+        <v>46315.5625</v>
       </c>
       <c r="B56">
-        <v>245</v>
+        <v>230</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="2">
-        <v>46310.57291666666</v>
+        <v>46315.57291666666</v>
       </c>
       <c r="B57">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="2">
-        <v>46310.58333333334</v>
+        <v>46315.58333333334</v>
       </c>
       <c r="B58">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="2">
-        <v>46310.59375</v>
+        <v>46315.59375</v>
       </c>
       <c r="B59">
-        <v>213</v>
+        <v>189</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="2">
-        <v>46310.60416666666</v>
+        <v>46315.60416666666</v>
       </c>
       <c r="B60">
-        <v>213</v>
+        <v>188</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="2">
-        <v>46310.61458333334</v>
+        <v>46315.61458333334</v>
       </c>
       <c r="B61">
-        <v>213</v>
+        <v>188</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="2">
-        <v>46310.625</v>
+        <v>46315.625</v>
       </c>
       <c r="B62">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="2">
-        <v>46310.63541666666</v>
+        <v>46315.63541666666</v>
       </c>
       <c r="B63">
         <v>226</v>
@@ -890,666 +890,554 @@
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2">
-        <v>46310.64583333334</v>
+        <v>46315.64583333334</v>
       </c>
       <c r="B64">
-        <v>209</v>
+        <v>227</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="2">
-        <v>46310.65625</v>
+        <v>46315.65625</v>
       </c>
       <c r="B65">
-        <v>259</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="2">
-        <v>46310.66666666666</v>
+        <v>46315.66666666666</v>
       </c>
       <c r="B66">
-        <v>603</v>
+        <v>467</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="2">
-        <v>46310.67708333334</v>
+        <v>46315.67708333334</v>
       </c>
       <c r="B67">
-        <v>652</v>
+        <v>471</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="2">
-        <v>46310.6875</v>
+        <v>46315.6875</v>
       </c>
       <c r="B68">
-        <v>632</v>
+        <v>473</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="2">
-        <v>46310.69791666666</v>
+        <v>46315.69791666666</v>
       </c>
       <c r="B69">
-        <v>633</v>
+        <v>480</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="2">
-        <v>46310.70833333334</v>
+        <v>46315.70833333334</v>
       </c>
       <c r="B70">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="2">
-        <v>46310.71875</v>
+        <v>46315.71875</v>
       </c>
       <c r="B71">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="2">
-        <v>46310.72916666666</v>
+        <v>46315.72916666666</v>
       </c>
       <c r="B72">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="2">
-        <v>46310.73958333334</v>
+        <v>46315.73958333334</v>
       </c>
       <c r="B73">
-        <v>710</v>
+        <v>672</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="2">
-        <v>46310.75</v>
+        <v>46315.75</v>
       </c>
       <c r="B74">
-        <v>689</v>
+        <v>671</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="2">
-        <v>46310.76041666666</v>
+        <v>46315.76041666666</v>
       </c>
       <c r="B75">
-        <v>692</v>
+        <v>669</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="2">
-        <v>46310.77083333334</v>
+        <v>46315.77083333334</v>
       </c>
       <c r="B76">
-        <v>678</v>
+        <v>660</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="2">
-        <v>46310.78125</v>
+        <v>46315.78125</v>
       </c>
       <c r="B77">
-        <v>678</v>
+        <v>660</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="2">
-        <v>46310.79166666666</v>
+        <v>46315.79166666666</v>
       </c>
       <c r="B78">
-        <v>687</v>
+        <v>665</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="2">
-        <v>46310.80208333334</v>
+        <v>46315.80208333334</v>
       </c>
       <c r="B79">
-        <v>687</v>
+        <v>663</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="2">
-        <v>46310.8125</v>
+        <v>46315.8125</v>
       </c>
       <c r="B80">
-        <v>687</v>
+        <v>664</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="2">
-        <v>46310.82291666666</v>
+        <v>46315.82291666666</v>
       </c>
       <c r="B81">
-        <v>688</v>
+        <v>638</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="2">
-        <v>46310.83333333334</v>
+        <v>46315.83333333334</v>
       </c>
       <c r="B82">
-        <v>682</v>
+        <v>677</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="2">
-        <v>46310.84375</v>
+        <v>46315.84375</v>
       </c>
       <c r="B83">
-        <v>677</v>
+        <v>717</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="2">
-        <v>46310.85416666666</v>
+        <v>46315.85416666666</v>
       </c>
       <c r="B84">
-        <v>677</v>
+        <v>717</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="2">
-        <v>46310.86458333334</v>
+        <v>46315.86458333334</v>
       </c>
       <c r="B85">
-        <v>658</v>
+        <v>680</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="2">
-        <v>46310.875</v>
+        <v>46315.875</v>
       </c>
       <c r="B86">
-        <v>638</v>
+        <v>706</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="2">
-        <v>46310.88541666666</v>
+        <v>46315.88541666666</v>
       </c>
       <c r="B87">
-        <v>637</v>
+        <v>708</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="2">
-        <v>46310.89583333334</v>
+        <v>46315.89583333334</v>
       </c>
       <c r="B88">
-        <v>637</v>
+        <v>688</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="2">
-        <v>46310.90625</v>
+        <v>46315.90625</v>
       </c>
       <c r="B89">
-        <v>650</v>
+        <v>686</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="2">
-        <v>46310.91666666666</v>
+        <v>46315.91666666666</v>
       </c>
       <c r="B90">
-        <v>550</v>
+        <v>666</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="2">
-        <v>46310.92708333334</v>
+        <v>46315.92708333334</v>
       </c>
       <c r="B91">
-        <v>527</v>
+        <v>661</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="2">
-        <v>46310.9375</v>
+        <v>46315.9375</v>
       </c>
       <c r="B92">
-        <v>527</v>
+        <v>662</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="2">
-        <v>46310.94791666666</v>
+        <v>46315.94791666666</v>
       </c>
       <c r="B93">
-        <v>525</v>
+        <v>660</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="2">
-        <v>46310.95833333334</v>
+        <v>46315.95833333334</v>
       </c>
       <c r="B94">
-        <v>452</v>
+        <v>627</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="2">
-        <v>46310.96875</v>
+        <v>46315.96875</v>
       </c>
       <c r="B95">
-        <v>441</v>
+        <v>558</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="2">
-        <v>46310.97916666666</v>
+        <v>46315.97916666666</v>
       </c>
       <c r="B96">
-        <v>441</v>
+        <v>582</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="2">
-        <v>46310.98958333334</v>
+        <v>46315.98958333334</v>
       </c>
       <c r="B97">
-        <v>439</v>
+        <v>572</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="2">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="B98">
-        <v>420</v>
+        <v>246</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="2">
-        <v>46311.01041666666</v>
+        <v>46316.01041666666</v>
       </c>
       <c r="B99">
-        <v>417</v>
+        <v>224</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="2">
-        <v>46311.02083333334</v>
+        <v>46316.02083333334</v>
       </c>
       <c r="B100">
-        <v>417</v>
+        <v>224</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="2">
-        <v>46311.03125</v>
+        <v>46316.03125</v>
       </c>
       <c r="B101">
-        <v>417</v>
+        <v>224</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="2">
-        <v>46311.04166666666</v>
+        <v>46316.04166666666</v>
       </c>
       <c r="B102">
-        <v>418</v>
+        <v>224</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="2">
-        <v>46311.05208333334</v>
+        <v>46316.05208333334</v>
       </c>
       <c r="B103">
-        <v>418</v>
+        <v>224</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="2">
-        <v>46311.0625</v>
+        <v>46316.0625</v>
       </c>
       <c r="B104">
-        <v>417</v>
+        <v>224</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="2">
-        <v>46311.07291666666</v>
+        <v>46316.07291666666</v>
       </c>
       <c r="B105">
-        <v>417</v>
+        <v>224</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="2">
-        <v>46311.08333333334</v>
+        <v>46316.08333333334</v>
       </c>
       <c r="B106">
-        <v>412</v>
+        <v>227</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="2">
-        <v>46311.09375</v>
+        <v>46316.09375</v>
       </c>
       <c r="B107">
-        <v>412</v>
+        <v>275</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="2">
-        <v>46311.10416666666</v>
+        <v>46316.10416666666</v>
       </c>
       <c r="B108">
-        <v>412</v>
+        <v>275</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="2">
-        <v>46311.11458333334</v>
+        <v>46316.11458333334</v>
       </c>
       <c r="B109">
-        <v>412</v>
+        <v>274</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="2">
-        <v>46311.125</v>
+        <v>46316.125</v>
       </c>
       <c r="B110">
-        <v>403</v>
+        <v>276</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="2">
-        <v>46311.13541666666</v>
+        <v>46316.13541666666</v>
       </c>
       <c r="B111">
-        <v>403</v>
+        <v>276</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="2">
-        <v>46311.14583333334</v>
+        <v>46316.14583333334</v>
       </c>
       <c r="B112">
-        <v>403</v>
+        <v>275</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="2">
-        <v>46311.15625</v>
+        <v>46316.15625</v>
       </c>
       <c r="B113">
-        <v>402</v>
+        <v>275</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="2">
-        <v>46311.16666666666</v>
+        <v>46316.16666666666</v>
       </c>
       <c r="B114">
-        <v>403</v>
+        <v>229</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="2">
-        <v>46311.17708333334</v>
+        <v>46316.17708333334</v>
       </c>
       <c r="B115">
-        <v>403</v>
+        <v>272</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="2">
-        <v>46311.1875</v>
+        <v>46316.1875</v>
       </c>
       <c r="B116">
-        <v>403</v>
+        <v>275</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="2">
-        <v>46311.19791666666</v>
+        <v>46316.19791666666</v>
       </c>
       <c r="B117">
-        <v>402</v>
+        <v>274</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="2">
-        <v>46311.20833333334</v>
+        <v>46316.20833333334</v>
       </c>
       <c r="B118">
-        <v>417</v>
+        <v>315</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="2">
-        <v>46311.21875</v>
+        <v>46316.21875</v>
       </c>
       <c r="B119">
-        <v>420</v>
+        <v>326</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="2">
-        <v>46311.22916666666</v>
+        <v>46316.22916666666</v>
       </c>
       <c r="B120">
-        <v>421</v>
+        <v>231</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="2">
-        <v>46311.23958333334</v>
+        <v>46316.23958333334</v>
       </c>
       <c r="B121">
-        <v>421</v>
+        <v>229</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="2">
-        <v>46311.25</v>
+        <v>46316.25</v>
       </c>
       <c r="B122">
-        <v>416</v>
+        <v>559</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="2">
-        <v>46311.26041666666</v>
+        <v>46316.26041666666</v>
       </c>
       <c r="B123">
-        <v>411</v>
+        <v>570</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="2">
-        <v>46311.27083333334</v>
+        <v>46316.27083333334</v>
       </c>
       <c r="B124">
-        <v>414</v>
+        <v>570</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="2">
-        <v>46311.28125</v>
+        <v>46316.28125</v>
       </c>
       <c r="B125">
-        <v>415</v>
+        <v>570</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="2">
-        <v>46311.29166666666</v>
+        <v>46316.29166666666</v>
       </c>
       <c r="B126">
-        <v>449</v>
+        <v>560</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="2">
-        <v>46311.30208333334</v>
+        <v>46316.30208333334</v>
       </c>
       <c r="B127">
-        <v>448</v>
+        <v>561</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="2">
-        <v>46311.3125</v>
+        <v>46316.3125</v>
       </c>
       <c r="B128">
-        <v>458</v>
+        <v>562</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="2">
-        <v>46311.32291666666</v>
+        <v>46316.32291666666</v>
       </c>
       <c r="B129">
-        <v>459</v>
+        <v>561</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="2">
-        <v>46311.33333333334</v>
+        <v>46316.33333333334</v>
       </c>
       <c r="B130">
-        <v>446</v>
+        <v>539</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="2">
-        <v>46311.34375</v>
+        <v>46316.34375</v>
       </c>
       <c r="B131">
-        <v>443</v>
+        <v>538</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" s="2">
-        <v>46311.35416666666</v>
+        <v>46316.35416666666</v>
       </c>
       <c r="B132">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2">
-      <c r="A133" s="2">
-        <v>46311.36458333334</v>
-      </c>
-      <c r="B133">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2">
-      <c r="A134" s="2">
-        <v>46311.375</v>
-      </c>
-      <c r="B134">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2">
-      <c r="A135" s="2">
-        <v>46311.38541666666</v>
-      </c>
-      <c r="B135">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2">
-      <c r="A136" s="2">
-        <v>46311.39583333334</v>
-      </c>
-      <c r="B136">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2">
-      <c r="A137" s="2">
-        <v>46311.40625</v>
-      </c>
-      <c r="B137">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2">
-      <c r="A138" s="2">
-        <v>46311.41666666666</v>
-      </c>
-      <c r="B138">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2">
-      <c r="A139" s="2">
-        <v>46311.42708333334</v>
-      </c>
-      <c r="B139">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2">
-      <c r="A140" s="2">
-        <v>46311.4375</v>
-      </c>
-      <c r="B140">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2">
-      <c r="A141" s="2">
-        <v>46311.44791666666</v>
-      </c>
-      <c r="B141">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2">
-      <c r="A142" s="2">
-        <v>46311.45833333334</v>
-      </c>
-      <c r="B142">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2">
-      <c r="A143" s="2">
-        <v>46311.46875</v>
-      </c>
-      <c r="B143">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2">
-      <c r="A144" s="2">
-        <v>46311.47916666666</v>
-      </c>
-      <c r="B144">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2">
-      <c r="A145" s="2">
-        <v>46311.48958333334</v>
-      </c>
-      <c r="B145">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2">
-      <c r="A146" s="2">
-        <v>46311.5</v>
-      </c>
-      <c r="B146">
-        <v>204</v>
+        <v>582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>